<commit_message>
refactor(enemy): 廢掉 dualBonus/counterBuff/counterStun/wrongPenalty.dmgScale ver -947
Ray：「連 JS 的欄位一起廢掉，讓他們三個跟一般怪一樣就好」
Ray：「完美反擊後那隻 3 秒不出手，邏輯本身就不對，空戰要靠反擊打傷害，
     他不出手怎麼反擊？」
Ray：「dualBonus → 只要船戰敵都吃這個就好了」

- counterStun 整條拿掉：那個「獎勵」會把玩家的輸出來源關掉，方向是反的。
- counterBuff 拿掉，完美反擊的獎勵只剩全域一套（tuning.atkBuffSeconds 3 秒 x2）。
  ⚠⚠ 順手修一個沉默的老 bug：defense 那一行是
    api.triggerAtkBuff(cb && cb.seconds ? cb.seconds : 2) —— 寫死的 2 繞過了
    全域的 3，所以實際行為一直是「四張老卡 5 秒、其餘所有怪 2 秒、沒有人吃到 3」。
    現在不傳參數，全部統一 3 秒（鐵律 7）。
- dualBonus 由逐卡欄位改成場次規則 tuning.shipDualBonus:0.2 —— 那不是「這隻怪的
  性質」而是「這種場次的性質」。飛行交棒的三條路都帶 ship:true → state.shipBattle。
  日後新增任何一隻飛行遭遇自動吃到，不必記得補欄位。
- wrongPenalty.dmgScale 移除（一張卡都沒在用，純清格式）。
- Excel 同步拿掉 delayPenalty.dmgScale/timeDelta 兩欄（46 欄）。

⚠ 保留 JS 的 delayPenalty.dmgScale/timeDelta：只有 witch 在用（0.5／-1），而
  timeDelta 是相對盤面 intervalLimit 的，換不成絕對值（每一盤的 intervalLimit 不同）。
  Excel 上不出現，要改直接改 enemies.js。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/enemies.xlsx
+++ b/tools/enemies.xlsx
@@ -1855,7 +1855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ58"/>
+  <dimension ref="A1:AT58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1889,27 +1889,21 @@
     <col width="13" customWidth="1" min="29" max="29"/>
     <col width="22" customWidth="1" min="30" max="30"/>
     <col width="21" customWidth="1" min="31" max="31"/>
-    <col width="23" customWidth="1" min="32" max="32"/>
-    <col width="24" customWidth="1" min="33" max="33"/>
-    <col width="16" customWidth="1" min="34" max="34"/>
-    <col width="16" customWidth="1" min="35" max="35"/>
-    <col width="18" customWidth="1" min="36" max="36"/>
-    <col width="9" customWidth="1" min="37" max="37"/>
-    <col width="20" customWidth="1" min="38" max="38"/>
-    <col width="46" customWidth="1" min="39" max="39"/>
-    <col width="10" customWidth="1" min="40" max="40"/>
-    <col width="15" customWidth="1" min="41" max="41"/>
-    <col width="17" customWidth="1" min="42" max="42"/>
-    <col width="9" customWidth="1" min="43" max="43"/>
-    <col width="27" customWidth="1" min="44" max="44"/>
-    <col width="11" customWidth="1" min="45" max="45"/>
-    <col width="21" customWidth="1" min="46" max="46"/>
-    <col width="23" customWidth="1" min="47" max="47"/>
-    <col width="46" customWidth="1" min="48" max="48"/>
-    <col width="25" customWidth="1" min="49" max="49"/>
-    <col width="11" customWidth="1" min="50" max="50"/>
-    <col width="27" customWidth="1" min="51" max="51"/>
-    <col width="13" customWidth="1" min="52" max="52"/>
+    <col width="16" customWidth="1" min="32" max="32"/>
+    <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="9" customWidth="1" min="35" max="35"/>
+    <col width="20" customWidth="1" min="36" max="36"/>
+    <col width="46" customWidth="1" min="37" max="37"/>
+    <col width="10" customWidth="1" min="38" max="38"/>
+    <col width="15" customWidth="1" min="39" max="39"/>
+    <col width="17" customWidth="1" min="40" max="40"/>
+    <col width="9" customWidth="1" min="41" max="41"/>
+    <col width="27" customWidth="1" min="42" max="42"/>
+    <col width="11" customWidth="1" min="43" max="43"/>
+    <col width="21" customWidth="1" min="44" max="44"/>
+    <col width="46" customWidth="1" min="45" max="45"/>
+    <col width="25" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2070,107 +2064,77 @@
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>delayPenalty.dmgScale</t>
+          <t>resist</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>delayPenalty.timeDelta</t>
+          <t>weak</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>resist</t>
+          <t>landSe</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>weak</t>
+          <t>special</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>landSe</t>
+          <t>boardGrids</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>special</t>
+          <t>hitFx</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>boardGrids</t>
+          <t>fit.mode</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>hitFx</t>
+          <t>fit.pos</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>fit.mode</t>
+          <t>entranceVo</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>fit.pos</t>
+          <t>noStack</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
         <is>
-          <t>entranceVo</t>
+          <t>bg</t>
         </is>
       </c>
       <c r="AQ1" s="1" t="inlineStr">
         <is>
-          <t>noStack</t>
+          <t>boardLoop</t>
         </is>
       </c>
       <c r="AR1" s="1" t="inlineStr">
         <is>
-          <t>bg</t>
+          <t>wrongPenalty.damage</t>
         </is>
       </c>
       <c r="AS1" s="1" t="inlineStr">
         <is>
-          <t>boardLoop</t>
+          <t>loot</t>
         </is>
       </c>
       <c r="AT1" s="1" t="inlineStr">
         <is>
-          <t>wrongPenalty.damage</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>wrongPenalty.dmgScale</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>loot</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
-        <is>
           <t>money</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
-        <is>
-          <t>dualBonus</t>
-        </is>
-      </c>
-      <c r="AY1" s="1" t="inlineStr">
-        <is>
-          <t>counterBuff</t>
-        </is>
-      </c>
-      <c r="AZ1" s="1" t="inlineStr">
-        <is>
-          <t>counterStun</t>
         </is>
       </c>
     </row>
@@ -2272,34 +2236,34 @@
         <v>5</v>
       </c>
       <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 9]</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
           <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "bite"}}</t>
         </is>
       </c>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr"/>
@@ -2307,12 +2271,6 @@
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
     </row>
     <row r="3" ht="49.92" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -2412,34 +2370,34 @@
         <v>5</v>
       </c>
       <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr"/>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 9]</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
           <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="inlineStr"/>
@@ -2447,12 +2405,6 @@
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr"/>
       <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
     </row>
     <row r="4" ht="62.40000000000001" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -2550,34 +2502,34 @@
       </c>
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 9]</t>
-        </is>
-      </c>
-      <c r="AM4" t="inlineStr">
-        <is>
           <t>{"delay": {"type": "slash"}, "wrong": {"type": "slash"}, "assault": {"type": "slash"}}</t>
         </is>
       </c>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="inlineStr"/>
       <c r="AP4" t="inlineStr"/>
@@ -2585,12 +2537,6 @@
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr"/>
       <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="inlineStr"/>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
     </row>
     <row r="5" ht="62.40000000000001" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -2688,34 +2634,34 @@
       </c>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL5" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 9]</t>
-        </is>
-      </c>
-      <c r="AM5" t="inlineStr">
-        <is>
           <t>{"delay": {"type": "slash"}, "wrong": {"type": "slash"}, "assault": {"type": "slash"}}</t>
         </is>
       </c>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
       <c r="AP5" t="inlineStr"/>
@@ -2723,12 +2669,6 @@
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="inlineStr"/>
       <c r="AT5" t="inlineStr"/>
-      <c r="AU5" t="inlineStr"/>
-      <c r="AV5" t="inlineStr"/>
-      <c r="AW5" t="inlineStr"/>
-      <c r="AX5" t="inlineStr"/>
-      <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="inlineStr"/>
     </row>
     <row r="6" ht="52.26000000000001" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -2830,51 +2770,45 @@
         <v>5</v>
       </c>
       <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr">
+      <c r="AF6" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL6" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 9]</t>
-        </is>
-      </c>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "bite"}}</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "bite"}}</t>
+          <t>62% 78%</t>
         </is>
       </c>
       <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>62% 78%</t>
-        </is>
-      </c>
+      <c r="AO6" t="inlineStr"/>
       <c r="AP6" t="inlineStr"/>
       <c r="AQ6" t="inlineStr"/>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="inlineStr"/>
       <c r="AT6" t="inlineStr"/>
-      <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
-      <c r="AX6" t="inlineStr"/>
-      <c r="AY6" t="inlineStr"/>
-      <c r="AZ6" t="inlineStr"/>
     </row>
     <row r="7" ht="74.88" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -2976,57 +2910,51 @@
         <v>4</v>
       </c>
       <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr">
+      <c r="AF7" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ7" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 16]</t>
+        </is>
+      </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL7" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 16]</t>
-        </is>
-      </c>
+          <t>{"delay": {"type": "dagger"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 4, "angle": "random"}}</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "dagger"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 4, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr">
-        <is>
           <t>50% 30%</t>
         </is>
       </c>
-      <c r="AP7" t="inlineStr">
+      <c r="AN7" t="inlineStr">
         <is>
           <t>vo_sorana_pack2</t>
         </is>
       </c>
-      <c r="AQ7" t="b">
-        <v>1</v>
-      </c>
+      <c r="AO7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
-      <c r="AX7" t="inlineStr"/>
-      <c r="AY7" t="inlineStr"/>
-      <c r="AZ7" t="inlineStr"/>
     </row>
     <row r="8" ht="74.88" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -3128,51 +3056,45 @@
         <v>5</v>
       </c>
       <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr">
+      <c r="AF8" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ8" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL8" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 9]</t>
-        </is>
-      </c>
+          <t>{"delay": {"type": "claw", "count": 4, "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "bite", "count": 4, "angle": "random"}}</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr"/>
       <c r="AM8" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "claw", "count": 4, "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "bite", "count": 4, "angle": "random"}}</t>
+          <t>50% 30%</t>
         </is>
       </c>
       <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr">
-        <is>
-          <t>50% 30%</t>
-        </is>
-      </c>
+      <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="inlineStr"/>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
-      <c r="AX8" t="inlineStr"/>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
     </row>
     <row r="9" ht="70.98" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -3268,34 +3190,34 @@
         <v>5</v>
       </c>
       <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr">
+      <c r="AF9" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ9" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL9" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 9]</t>
-        </is>
-      </c>
-      <c r="AM9" t="inlineStr">
-        <is>
           <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "bite"}}</t>
         </is>
       </c>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
@@ -3303,12 +3225,6 @@
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="inlineStr"/>
       <c r="AT9" t="inlineStr"/>
-      <c r="AU9" t="inlineStr"/>
-      <c r="AV9" t="inlineStr"/>
-      <c r="AW9" t="inlineStr"/>
-      <c r="AX9" t="inlineStr"/>
-      <c r="AY9" t="inlineStr"/>
-      <c r="AZ9" t="inlineStr"/>
     </row>
     <row r="10" ht="62.40000000000001" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -3406,38 +3322,34 @@
       </c>
       <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AG10" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AH10" t="inlineStr">
+      <c r="AF10" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ10" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>[9, 9, 16, 16, 16]</t>
+        </is>
+      </c>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL10" t="inlineStr">
-        <is>
-          <t>[9, 9, 16, 16, 16]</t>
-        </is>
-      </c>
-      <c r="AM10" t="inlineStr">
-        <is>
           <t>{"delay": {"type": "bullet", "count": 1, "pos": "random"}, "wrong": {"type": "dagger"}, "assault": {"type": "witch_revolver", "count": 1, "pos": "random", "scale": 1.6}}</t>
         </is>
       </c>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
@@ -3445,12 +3357,6 @@
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
       <c r="AT10" t="inlineStr"/>
-      <c r="AU10" t="inlineStr"/>
-      <c r="AV10" t="inlineStr"/>
-      <c r="AW10" t="inlineStr"/>
-      <c r="AX10" t="inlineStr"/>
-      <c r="AY10" t="inlineStr"/>
-      <c r="AZ10" t="inlineStr"/>
     </row>
     <row r="11" ht="74.10000000000001" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -3550,59 +3456,53 @@
         <v>6</v>
       </c>
       <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="inlineStr">
+      <c r="AF11" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ11" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL11" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM11" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN11" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO11" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>Northport_church_BF</t>
+        </is>
+      </c>
       <c r="AQ11" t="inlineStr"/>
-      <c r="AR11" t="inlineStr">
-        <is>
-          <t>Northport_church_BF</t>
-        </is>
-      </c>
+      <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr"/>
       <c r="AT11" t="inlineStr"/>
-      <c r="AU11" t="inlineStr"/>
-      <c r="AV11" t="inlineStr"/>
-      <c r="AW11" t="inlineStr"/>
-      <c r="AX11" t="inlineStr"/>
-      <c r="AY11" t="inlineStr"/>
-      <c r="AZ11" t="inlineStr"/>
     </row>
     <row r="12" ht="74.88" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -3702,59 +3602,53 @@
         <v>5</v>
       </c>
       <c r="AE12" t="inlineStr"/>
-      <c r="AF12" t="inlineStr"/>
-      <c r="AG12" t="inlineStr"/>
-      <c r="AH12" t="inlineStr">
+      <c r="AF12" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr"/>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ12" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM12" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN12" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO12" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>Northport_church_BF</t>
+        </is>
+      </c>
       <c r="AQ12" t="inlineStr"/>
-      <c r="AR12" t="inlineStr">
-        <is>
-          <t>Northport_church_BF</t>
-        </is>
-      </c>
+      <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
       <c r="AT12" t="inlineStr"/>
-      <c r="AU12" t="inlineStr"/>
-      <c r="AV12" t="inlineStr"/>
-      <c r="AW12" t="inlineStr"/>
-      <c r="AX12" t="inlineStr"/>
-      <c r="AY12" t="inlineStr"/>
-      <c r="AZ12" t="inlineStr"/>
     </row>
     <row r="13" ht="74.88" customHeight="1">
       <c r="A13" t="inlineStr">
@@ -3854,59 +3748,53 @@
         <v>5</v>
       </c>
       <c r="AE13" t="inlineStr"/>
-      <c r="AF13" t="inlineStr"/>
-      <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr">
+      <c r="AF13" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ13" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL13" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM13" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN13" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO13" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP13" t="inlineStr"/>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>Northport_church_BF</t>
+        </is>
+      </c>
       <c r="AQ13" t="inlineStr"/>
-      <c r="AR13" t="inlineStr">
-        <is>
-          <t>Northport_church_BF</t>
-        </is>
-      </c>
+      <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
       <c r="AT13" t="inlineStr"/>
-      <c r="AU13" t="inlineStr"/>
-      <c r="AV13" t="inlineStr"/>
-      <c r="AW13" t="inlineStr"/>
-      <c r="AX13" t="inlineStr"/>
-      <c r="AY13" t="inlineStr"/>
-      <c r="AZ13" t="inlineStr"/>
     </row>
     <row r="14" ht="74.10000000000001" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -4006,59 +3894,53 @@
         <v>5</v>
       </c>
       <c r="AE14" t="inlineStr"/>
-      <c r="AF14" t="inlineStr"/>
-      <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr">
+      <c r="AF14" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr"/>
       <c r="AI14" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ14" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL14" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM14" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN14" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO14" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP14" t="inlineStr"/>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>Northport_church_BF</t>
+        </is>
+      </c>
       <c r="AQ14" t="inlineStr"/>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>Northport_church_BF</t>
-        </is>
-      </c>
+      <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
       <c r="AT14" t="inlineStr"/>
-      <c r="AU14" t="inlineStr"/>
-      <c r="AV14" t="inlineStr"/>
-      <c r="AW14" t="inlineStr"/>
-      <c r="AX14" t="inlineStr"/>
-      <c r="AY14" t="inlineStr"/>
-      <c r="AZ14" t="inlineStr"/>
     </row>
     <row r="15" ht="74.88" customHeight="1">
       <c r="A15" t="inlineStr">
@@ -4158,59 +4040,53 @@
         <v>6</v>
       </c>
       <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr">
+      <c r="AF15" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr"/>
       <c r="AI15" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ15" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "blood", "angle": "random"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL15" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM15" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "blood", "angle": "random"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN15" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO15" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP15" t="inlineStr"/>
+      <c r="AN15" t="inlineStr"/>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>Northport_church_BF</t>
+        </is>
+      </c>
       <c r="AQ15" t="inlineStr"/>
-      <c r="AR15" t="inlineStr">
-        <is>
-          <t>Northport_church_BF</t>
-        </is>
-      </c>
+      <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="inlineStr"/>
       <c r="AT15" t="inlineStr"/>
-      <c r="AU15" t="inlineStr"/>
-      <c r="AV15" t="inlineStr"/>
-      <c r="AW15" t="inlineStr"/>
-      <c r="AX15" t="inlineStr"/>
-      <c r="AY15" t="inlineStr"/>
-      <c r="AZ15" t="inlineStr"/>
     </row>
     <row r="16" ht="49.92" customHeight="1">
       <c r="A16" t="inlineStr">
@@ -4310,51 +4186,45 @@
         <v>5</v>
       </c>
       <c r="AE16" t="inlineStr"/>
-      <c r="AF16" t="inlineStr"/>
-      <c r="AG16" t="inlineStr"/>
-      <c r="AH16" t="inlineStr">
+      <c r="AF16" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr"/>
       <c r="AI16" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ16" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 16]</t>
+        </is>
+      </c>
       <c r="AK16" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL16" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 16]</t>
-        </is>
-      </c>
-      <c r="AM16" t="inlineStr">
-        <is>
           <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="inlineStr"/>
       <c r="AN16" t="inlineStr"/>
       <c r="AO16" t="inlineStr"/>
-      <c r="AP16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Northport_church_BF</t>
+        </is>
+      </c>
       <c r="AQ16" t="inlineStr"/>
-      <c r="AR16" t="inlineStr">
-        <is>
-          <t>Northport_church_BF</t>
-        </is>
-      </c>
+      <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="inlineStr"/>
       <c r="AT16" t="inlineStr"/>
-      <c r="AU16" t="inlineStr"/>
-      <c r="AV16" t="inlineStr"/>
-      <c r="AW16" t="inlineStr"/>
-      <c r="AX16" t="inlineStr"/>
-      <c r="AY16" t="inlineStr"/>
-      <c r="AZ16" t="inlineStr"/>
     </row>
     <row r="17" ht="74.88" customHeight="1">
       <c r="A17" t="inlineStr">
@@ -4454,59 +4324,53 @@
         <v>5</v>
       </c>
       <c r="AE17" t="inlineStr"/>
-      <c r="AF17" t="inlineStr"/>
-      <c r="AG17" t="inlineStr"/>
-      <c r="AH17" t="inlineStr">
+      <c r="AF17" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr"/>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ17" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL17" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM17" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN17" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO17" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP17" t="inlineStr"/>
+      <c r="AN17" t="inlineStr"/>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>Shinier_North</t>
+        </is>
+      </c>
       <c r="AQ17" t="inlineStr"/>
-      <c r="AR17" t="inlineStr">
-        <is>
-          <t>Shinier_North</t>
-        </is>
-      </c>
+      <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="inlineStr"/>
       <c r="AT17" t="inlineStr"/>
-      <c r="AU17" t="inlineStr"/>
-      <c r="AV17" t="inlineStr"/>
-      <c r="AW17" t="inlineStr"/>
-      <c r="AX17" t="inlineStr"/>
-      <c r="AY17" t="inlineStr"/>
-      <c r="AZ17" t="inlineStr"/>
     </row>
     <row r="18" ht="74.10000000000001" customHeight="1">
       <c r="A18" t="inlineStr">
@@ -4606,59 +4470,53 @@
         <v>5</v>
       </c>
       <c r="AE18" t="inlineStr"/>
-      <c r="AF18" t="inlineStr"/>
-      <c r="AG18" t="inlineStr"/>
-      <c r="AH18" t="inlineStr">
+      <c r="AF18" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr"/>
       <c r="AI18" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ18" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM18" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN18" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO18" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP18" t="inlineStr"/>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>Shinier_North</t>
+        </is>
+      </c>
       <c r="AQ18" t="inlineStr"/>
-      <c r="AR18" t="inlineStr">
-        <is>
-          <t>Shinier_North</t>
-        </is>
-      </c>
+      <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="inlineStr"/>
       <c r="AT18" t="inlineStr"/>
-      <c r="AU18" t="inlineStr"/>
-      <c r="AV18" t="inlineStr"/>
-      <c r="AW18" t="inlineStr"/>
-      <c r="AX18" t="inlineStr"/>
-      <c r="AY18" t="inlineStr"/>
-      <c r="AZ18" t="inlineStr"/>
     </row>
     <row r="19" ht="42.12" customHeight="1">
       <c r="A19" t="inlineStr">
@@ -4758,59 +4616,53 @@
         <v>5</v>
       </c>
       <c r="AE19" t="inlineStr"/>
-      <c r="AF19" t="inlineStr"/>
-      <c r="AG19" t="inlineStr"/>
-      <c r="AH19" t="inlineStr">
+      <c r="AF19" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr"/>
       <c r="AI19" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ19" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL19" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM19" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN19" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO19" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP19" t="inlineStr"/>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>Shinier_North</t>
+        </is>
+      </c>
       <c r="AQ19" t="inlineStr"/>
-      <c r="AR19" t="inlineStr">
-        <is>
-          <t>Shinier_North</t>
-        </is>
-      </c>
+      <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="inlineStr"/>
       <c r="AT19" t="inlineStr"/>
-      <c r="AU19" t="inlineStr"/>
-      <c r="AV19" t="inlineStr"/>
-      <c r="AW19" t="inlineStr"/>
-      <c r="AX19" t="inlineStr"/>
-      <c r="AY19" t="inlineStr"/>
-      <c r="AZ19" t="inlineStr"/>
     </row>
     <row r="20" ht="74.88" customHeight="1">
       <c r="A20" t="inlineStr">
@@ -4910,59 +4762,53 @@
         <v>5</v>
       </c>
       <c r="AE20" t="inlineStr"/>
-      <c r="AF20" t="inlineStr"/>
-      <c r="AG20" t="inlineStr"/>
-      <c r="AH20" t="inlineStr">
+      <c r="AF20" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr"/>
       <c r="AI20" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ20" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL20" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM20" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN20" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO20" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP20" t="inlineStr"/>
+      <c r="AN20" t="inlineStr"/>
+      <c r="AO20" t="inlineStr"/>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>Shinier_North</t>
+        </is>
+      </c>
       <c r="AQ20" t="inlineStr"/>
-      <c r="AR20" t="inlineStr">
-        <is>
-          <t>Shinier_North</t>
-        </is>
-      </c>
+      <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="inlineStr"/>
       <c r="AT20" t="inlineStr"/>
-      <c r="AU20" t="inlineStr"/>
-      <c r="AV20" t="inlineStr"/>
-      <c r="AW20" t="inlineStr"/>
-      <c r="AX20" t="inlineStr"/>
-      <c r="AY20" t="inlineStr"/>
-      <c r="AZ20" t="inlineStr"/>
     </row>
     <row r="21" ht="51.48" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -5062,59 +4908,53 @@
         <v>6</v>
       </c>
       <c r="AE21" t="inlineStr"/>
-      <c r="AF21" t="inlineStr"/>
-      <c r="AG21" t="inlineStr"/>
-      <c r="AH21" t="inlineStr">
+      <c r="AF21" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr"/>
       <c r="AI21" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ21" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK21" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL21" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM21" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN21" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO21" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP21" t="inlineStr"/>
+      <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>Shinier_Wilds</t>
+        </is>
+      </c>
       <c r="AQ21" t="inlineStr"/>
-      <c r="AR21" t="inlineStr">
-        <is>
-          <t>Shinier_Wilds</t>
-        </is>
-      </c>
+      <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="inlineStr"/>
       <c r="AT21" t="inlineStr"/>
-      <c r="AU21" t="inlineStr"/>
-      <c r="AV21" t="inlineStr"/>
-      <c r="AW21" t="inlineStr"/>
-      <c r="AX21" t="inlineStr"/>
-      <c r="AY21" t="inlineStr"/>
-      <c r="AZ21" t="inlineStr"/>
     </row>
     <row r="22" ht="74.88" customHeight="1">
       <c r="A22" t="inlineStr">
@@ -5214,59 +5054,53 @@
         <v>6</v>
       </c>
       <c r="AE22" t="inlineStr"/>
-      <c r="AF22" t="inlineStr"/>
-      <c r="AG22" t="inlineStr"/>
-      <c r="AH22" t="inlineStr">
+      <c r="AF22" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr"/>
       <c r="AI22" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ22" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK22" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "blood", "angle": "random"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL22" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM22" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "blood", "angle": "random"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN22" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO22" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP22" t="inlineStr"/>
+      <c r="AN22" t="inlineStr"/>
+      <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>Shinier_Altar</t>
+        </is>
+      </c>
       <c r="AQ22" t="inlineStr"/>
-      <c r="AR22" t="inlineStr">
-        <is>
-          <t>Shinier_Altar</t>
-        </is>
-      </c>
+      <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="inlineStr"/>
       <c r="AT22" t="inlineStr"/>
-      <c r="AU22" t="inlineStr"/>
-      <c r="AV22" t="inlineStr"/>
-      <c r="AW22" t="inlineStr"/>
-      <c r="AX22" t="inlineStr"/>
-      <c r="AY22" t="inlineStr"/>
-      <c r="AZ22" t="inlineStr"/>
     </row>
     <row r="23" ht="74.88" customHeight="1">
       <c r="A23" t="inlineStr">
@@ -5368,71 +5202,65 @@
       <c r="AE23" t="n">
         <v>5</v>
       </c>
-      <c r="AF23" t="inlineStr"/>
-      <c r="AG23" t="inlineStr"/>
-      <c r="AH23" t="inlineStr">
+      <c r="AF23" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr"/>
       <c r="AI23" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AJ23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK23" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "bullet", "count": 1, "pos": "random"}, "wrong": {"type": "blunt"}, "assault": {"type": "bullet", "count": 1, "pos": "random", "scale": 1.8}}</t>
         </is>
       </c>
       <c r="AL23" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM23" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "bullet", "count": 1, "pos": "random"}, "wrong": {"type": "blunt"}, "assault": {"type": "bullet", "count": 1, "pos": "random", "scale": 1.8}}</t>
-        </is>
-      </c>
-      <c r="AN23" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO23" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP23" t="inlineStr"/>
-      <c r="AQ23" t="inlineStr"/>
-      <c r="AR23" t="inlineStr">
+      <c r="AN23" t="inlineStr"/>
+      <c r="AO23" t="inlineStr"/>
+      <c r="AP23" t="inlineStr">
         <is>
           <t>Captal_Guild_Day</t>
         </is>
       </c>
-      <c r="AS23" t="b">
-        <v>1</v>
-      </c>
-      <c r="AT23" t="n">
+      <c r="AQ23" t="b">
+        <v>1</v>
+      </c>
+      <c r="AR23" t="n">
         <v>5</v>
       </c>
-      <c r="AU23" t="inlineStr"/>
-      <c r="AV23" t="inlineStr">
+      <c r="AS23" t="inlineStr">
         <is>
           <t>[{"id": "brass_casing", "n": 6}]</t>
         </is>
       </c>
-      <c r="AW23" t="inlineStr">
+      <c r="AT23" t="inlineStr">
         <is>
           <t>{"hpRatio": [0.6, 0.8]}</t>
         </is>
       </c>
-      <c r="AX23" t="inlineStr"/>
-      <c r="AY23" t="inlineStr"/>
-      <c r="AZ23" t="inlineStr"/>
     </row>
     <row r="24" ht="66.3" customHeight="1">
       <c r="A24" t="inlineStr">
@@ -5534,72 +5362,58 @@
       <c r="AE24" t="n">
         <v>10</v>
       </c>
-      <c r="AF24" t="inlineStr"/>
-      <c r="AG24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>{"basic": 0.2}</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>{"counter": 1}</t>
+        </is>
+      </c>
       <c r="AH24" t="inlineStr">
         <is>
-          <t>{"basic": 0.2}</t>
+          <t>se_enemy_centipi</t>
         </is>
       </c>
       <c r="AI24" t="inlineStr">
         <is>
-          <t>{"counter": 1}</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>se_enemy_centipi</t>
+          <t>[9, 9, 9, 9, 16]</t>
         </is>
       </c>
       <c r="AK24" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL24" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 16]</t>
-        </is>
-      </c>
-      <c r="AM24" t="inlineStr">
-        <is>
           <t>{"delay": {"type": "claw", "count": 1, "angle": "random"}, "wrong": {"type": "blunt"}, "assault": {"type": "centipi_claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
+      <c r="AL24" t="inlineStr"/>
+      <c r="AM24" t="inlineStr"/>
       <c r="AN24" t="inlineStr"/>
-      <c r="AO24" t="inlineStr"/>
+      <c r="AO24" t="b">
+        <v>1</v>
+      </c>
       <c r="AP24" t="inlineStr"/>
       <c r="AQ24" t="b">
         <v>1</v>
       </c>
-      <c r="AR24" t="inlineStr"/>
-      <c r="AS24" t="b">
-        <v>1</v>
-      </c>
-      <c r="AT24" t="n">
+      <c r="AR24" t="n">
         <v>5</v>
       </c>
-      <c r="AU24" t="inlineStr"/>
-      <c r="AV24" t="inlineStr">
+      <c r="AS24" t="inlineStr">
         <is>
           <t>[{"id": "venom_fang", "n": 1, "p": 0.1}, {"id": "venom_claw", "n": 1, "p": 0.33}, {"id": "chitin_wing", "n": 1, "p": 0.1}, {"id": "chitin_shell", "n": 1, "p": 0.33}]</t>
         </is>
       </c>
-      <c r="AW24" t="inlineStr">
+      <c r="AT24" t="inlineStr">
         <is>
           <t>{"hpRatio": [1.2, 1.5]}</t>
         </is>
-      </c>
-      <c r="AX24" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AY24" t="inlineStr">
-        <is>
-          <t>{"mult": 2, "seconds": 5}</t>
-        </is>
-      </c>
-      <c r="AZ24" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="25" ht="39.78" customHeight="1">
@@ -5704,72 +5518,58 @@
       <c r="AE25" t="n">
         <v>10</v>
       </c>
-      <c r="AF25" t="inlineStr"/>
-      <c r="AG25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>{"basic": 0.2}</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>{"counter": 1}</t>
+        </is>
+      </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>{"basic": 0.2}</t>
+          <t>se_enemy_serpent</t>
         </is>
       </c>
       <c r="AI25" t="inlineStr">
         <is>
-          <t>{"counter": 1}</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>se_enemy_serpent</t>
+          <t>[9, 9, 9, 9, 16]</t>
         </is>
       </c>
       <c r="AK25" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL25" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 16]</t>
-        </is>
-      </c>
-      <c r="AM25" t="inlineStr">
-        <is>
           <t>{"delay": {"type": "claw", "count": 1, "angle": "random"}, "wrong": {"type": "blunt"}, "assault": {"type": "serpent_bite"}}</t>
         </is>
       </c>
+      <c r="AL25" t="inlineStr"/>
+      <c r="AM25" t="inlineStr"/>
       <c r="AN25" t="inlineStr"/>
-      <c r="AO25" t="inlineStr"/>
+      <c r="AO25" t="b">
+        <v>1</v>
+      </c>
       <c r="AP25" t="inlineStr"/>
       <c r="AQ25" t="b">
         <v>1</v>
       </c>
-      <c r="AR25" t="inlineStr"/>
-      <c r="AS25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AT25" t="n">
+      <c r="AR25" t="n">
         <v>5</v>
       </c>
-      <c r="AU25" t="inlineStr"/>
-      <c r="AV25" t="inlineStr">
+      <c r="AS25" t="inlineStr">
         <is>
           <t>[{"id": "venom_fang", "n": 1, "p": 0.1}, {"id": "azure_scale", "n": 1, "p": 0.33}, {"id": "azure_feather", "n": 1, "p": 0.33}]</t>
         </is>
       </c>
-      <c r="AW25" t="inlineStr">
+      <c r="AT25" t="inlineStr">
         <is>
           <t>{"hpRatio": [0.5, 0.7]}</t>
         </is>
-      </c>
-      <c r="AX25" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AY25" t="inlineStr">
-        <is>
-          <t>{"mult": 2, "seconds": 5}</t>
-        </is>
-      </c>
-      <c r="AZ25" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="26" ht="33.54" customHeight="1">
@@ -5874,72 +5674,58 @@
       <c r="AE26" t="n">
         <v>10</v>
       </c>
-      <c r="AF26" t="inlineStr"/>
-      <c r="AG26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>{"basic": 0.2}</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>{"counter": 1}</t>
+        </is>
+      </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>{"basic": 0.2}</t>
+          <t>se_weapon_cannon</t>
         </is>
       </c>
       <c r="AI26" t="inlineStr">
         <is>
-          <t>{"counter": 1}</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
-          <t>se_weapon_cannon</t>
+          <t>[9, 9, 9, 9, 16]</t>
         </is>
       </c>
       <c r="AK26" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AL26" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 16]</t>
-        </is>
-      </c>
-      <c r="AM26" t="inlineStr">
-        <is>
           <t>{"delay": {"type": "pirate_shipcannon", "count": 1, "pos": "random"}, "wrong": {"type": "pirate_sniper", "count": 1, "pos": "random"}, "assault": {"type": "pirate_cannon", "count": 1, "pos": "random", "scale": 2.4, "flash": "red"}}</t>
         </is>
       </c>
+      <c r="AL26" t="inlineStr"/>
+      <c r="AM26" t="inlineStr"/>
       <c r="AN26" t="inlineStr"/>
-      <c r="AO26" t="inlineStr"/>
+      <c r="AO26" t="b">
+        <v>1</v>
+      </c>
       <c r="AP26" t="inlineStr"/>
       <c r="AQ26" t="b">
         <v>1</v>
       </c>
-      <c r="AR26" t="inlineStr"/>
-      <c r="AS26" t="b">
-        <v>1</v>
-      </c>
-      <c r="AT26" t="n">
+      <c r="AR26" t="n">
         <v>5</v>
       </c>
-      <c r="AU26" t="inlineStr"/>
-      <c r="AV26" t="inlineStr">
+      <c r="AS26" t="inlineStr">
         <is>
           <t>[{"id": "brass_casing", "n": 1, "p": 0.33}]</t>
         </is>
       </c>
-      <c r="AW26" t="inlineStr">
+      <c r="AT26" t="inlineStr">
         <is>
           <t>{"hpRatio": [0.7, 0.9]}</t>
         </is>
-      </c>
-      <c r="AX26" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AY26" t="inlineStr">
-        <is>
-          <t>{"mult": 2, "seconds": 5}</t>
-        </is>
-      </c>
-      <c r="AZ26" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="27" ht="74.88" customHeight="1">
@@ -6040,63 +5826,57 @@
         <v>5</v>
       </c>
       <c r="AE27" t="inlineStr"/>
-      <c r="AF27" t="inlineStr"/>
-      <c r="AG27" t="inlineStr"/>
-      <c r="AH27" t="inlineStr">
+      <c r="AF27" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr"/>
       <c r="AI27" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ27" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK27" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "claw", "count": 1, "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "bite", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL27" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM27" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "claw", "count": 1, "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "bite", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN27" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO27" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP27" t="inlineStr"/>
+      <c r="AN27" t="inlineStr"/>
+      <c r="AO27" t="inlineStr"/>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>Forest_Glade_Day</t>
+        </is>
+      </c>
       <c r="AQ27" t="inlineStr"/>
-      <c r="AR27" t="inlineStr">
-        <is>
-          <t>Forest_Glade_Day</t>
-        </is>
-      </c>
-      <c r="AS27" t="inlineStr"/>
+      <c r="AR27" t="inlineStr"/>
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>[{"id": "meat_lynx", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT27" t="inlineStr"/>
-      <c r="AU27" t="inlineStr"/>
-      <c r="AV27" t="inlineStr">
-        <is>
-          <t>[{"id": "meat_lynx", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW27" t="inlineStr"/>
-      <c r="AX27" t="inlineStr"/>
-      <c r="AY27" t="inlineStr"/>
-      <c r="AZ27" t="inlineStr"/>
     </row>
     <row r="28" ht="74.10000000000001" customHeight="1">
       <c r="A28" t="inlineStr">
@@ -6196,63 +5976,57 @@
         <v>5</v>
       </c>
       <c r="AE28" t="inlineStr"/>
-      <c r="AF28" t="inlineStr"/>
-      <c r="AG28" t="inlineStr"/>
-      <c r="AH28" t="inlineStr">
+      <c r="AF28" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH28" t="inlineStr"/>
       <c r="AI28" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ28" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK28" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "bite"}, "wrong": {"type": "slash"}, "assault": {"type": "bite"}}</t>
         </is>
       </c>
       <c r="AL28" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM28" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "bite"}, "wrong": {"type": "slash"}, "assault": {"type": "bite"}}</t>
-        </is>
-      </c>
-      <c r="AN28" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO28" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP28" t="inlineStr"/>
+      <c r="AN28" t="inlineStr"/>
+      <c r="AO28" t="inlineStr"/>
+      <c r="AP28" t="inlineStr">
+        <is>
+          <t>Forest_Shoal_Day</t>
+        </is>
+      </c>
       <c r="AQ28" t="inlineStr"/>
-      <c r="AR28" t="inlineStr">
-        <is>
-          <t>Forest_Shoal_Day</t>
-        </is>
-      </c>
-      <c r="AS28" t="inlineStr"/>
+      <c r="AR28" t="inlineStr"/>
+      <c r="AS28" t="inlineStr">
+        <is>
+          <t>[{"id": "meat_snake", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT28" t="inlineStr"/>
-      <c r="AU28" t="inlineStr"/>
-      <c r="AV28" t="inlineStr">
-        <is>
-          <t>[{"id": "meat_snake", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW28" t="inlineStr"/>
-      <c r="AX28" t="inlineStr"/>
-      <c r="AY28" t="inlineStr"/>
-      <c r="AZ28" t="inlineStr"/>
     </row>
     <row r="29" ht="33.54" customHeight="1">
       <c r="A29" t="inlineStr">
@@ -6352,63 +6126,57 @@
         <v>5</v>
       </c>
       <c r="AE29" t="inlineStr"/>
-      <c r="AF29" t="inlineStr"/>
-      <c r="AG29" t="inlineStr"/>
-      <c r="AH29" t="inlineStr">
+      <c r="AF29" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH29" t="inlineStr"/>
       <c r="AI29" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ29" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK29" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL29" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM29" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN29" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO29" t="inlineStr">
-        <is>
           <t>center 70%</t>
         </is>
       </c>
-      <c r="AP29" t="inlineStr"/>
+      <c r="AN29" t="inlineStr"/>
+      <c r="AO29" t="inlineStr"/>
+      <c r="AP29" t="inlineStr">
+        <is>
+          <t>Forest_Trail_Day</t>
+        </is>
+      </c>
       <c r="AQ29" t="inlineStr"/>
-      <c r="AR29" t="inlineStr">
-        <is>
-          <t>Forest_Trail_Day</t>
-        </is>
-      </c>
-      <c r="AS29" t="inlineStr"/>
+      <c r="AR29" t="inlineStr"/>
+      <c r="AS29" t="inlineStr">
+        <is>
+          <t>[{"id": "meat_boar", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT29" t="inlineStr"/>
-      <c r="AU29" t="inlineStr"/>
-      <c r="AV29" t="inlineStr">
-        <is>
-          <t>[{"id": "meat_boar", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW29" t="inlineStr"/>
-      <c r="AX29" t="inlineStr"/>
-      <c r="AY29" t="inlineStr"/>
-      <c r="AZ29" t="inlineStr"/>
     </row>
     <row r="30" ht="33.54" customHeight="1">
       <c r="A30" t="inlineStr">
@@ -6508,63 +6276,57 @@
         <v>5</v>
       </c>
       <c r="AE30" t="inlineStr"/>
-      <c r="AF30" t="inlineStr"/>
-      <c r="AG30" t="inlineStr"/>
-      <c r="AH30" t="inlineStr">
+      <c r="AF30" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH30" t="inlineStr"/>
       <c r="AI30" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ30" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK30" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "claw", "count": 1, "angle": "random"}, "wrong": {"type": "bite"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL30" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM30" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "claw", "count": 1, "angle": "random"}, "wrong": {"type": "bite"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN30" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO30" t="inlineStr">
-        <is>
           <t>center 55%</t>
         </is>
       </c>
-      <c r="AP30" t="inlineStr"/>
+      <c r="AN30" t="inlineStr"/>
+      <c r="AO30" t="inlineStr"/>
+      <c r="AP30" t="inlineStr">
+        <is>
+          <t>Forest_Cave_Day</t>
+        </is>
+      </c>
       <c r="AQ30" t="inlineStr"/>
-      <c r="AR30" t="inlineStr">
-        <is>
-          <t>Forest_Cave_Day</t>
-        </is>
-      </c>
-      <c r="AS30" t="inlineStr"/>
+      <c r="AR30" t="inlineStr"/>
+      <c r="AS30" t="inlineStr">
+        <is>
+          <t>[{"id": "tiger_horn", "n": 1, "p": 0.25}]</t>
+        </is>
+      </c>
       <c r="AT30" t="inlineStr"/>
-      <c r="AU30" t="inlineStr"/>
-      <c r="AV30" t="inlineStr">
-        <is>
-          <t>[{"id": "tiger_horn", "n": 1, "p": 0.25}]</t>
-        </is>
-      </c>
-      <c r="AW30" t="inlineStr"/>
-      <c r="AX30" t="inlineStr"/>
-      <c r="AY30" t="inlineStr"/>
-      <c r="AZ30" t="inlineStr"/>
     </row>
     <row r="31" ht="74.88" customHeight="1">
       <c r="A31" t="inlineStr">
@@ -6664,63 +6426,57 @@
         <v>5</v>
       </c>
       <c r="AE31" t="inlineStr"/>
-      <c r="AF31" t="inlineStr"/>
-      <c r="AG31" t="inlineStr"/>
-      <c r="AH31" t="inlineStr">
+      <c r="AF31" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH31" t="inlineStr"/>
       <c r="AI31" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ31" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK31" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "slash"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL31" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM31" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "slash"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN31" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO31" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP31" t="inlineStr"/>
+      <c r="AN31" t="inlineStr"/>
+      <c r="AO31" t="inlineStr"/>
+      <c r="AP31" t="inlineStr">
+        <is>
+          <t>Forest_Glade_Day</t>
+        </is>
+      </c>
       <c r="AQ31" t="inlineStr"/>
-      <c r="AR31" t="inlineStr">
-        <is>
-          <t>Forest_Glade_Day</t>
-        </is>
-      </c>
-      <c r="AS31" t="inlineStr"/>
+      <c r="AR31" t="inlineStr"/>
+      <c r="AS31" t="inlineStr">
+        <is>
+          <t>[{"id": "crow_beak", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT31" t="inlineStr"/>
-      <c r="AU31" t="inlineStr"/>
-      <c r="AV31" t="inlineStr">
-        <is>
-          <t>[{"id": "crow_beak", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW31" t="inlineStr"/>
-      <c r="AX31" t="inlineStr"/>
-      <c r="AY31" t="inlineStr"/>
-      <c r="AZ31" t="inlineStr"/>
     </row>
     <row r="32" ht="53.04" customHeight="1">
       <c r="A32" t="inlineStr">
@@ -6820,63 +6576,57 @@
         <v>5</v>
       </c>
       <c r="AE32" t="inlineStr"/>
-      <c r="AF32" t="inlineStr"/>
-      <c r="AG32" t="inlineStr"/>
-      <c r="AH32" t="inlineStr">
+      <c r="AF32" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH32" t="inlineStr"/>
       <c r="AI32" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ32" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK32" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "sakura"}}</t>
         </is>
       </c>
       <c r="AL32" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM32" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "sakura"}}</t>
-        </is>
-      </c>
-      <c r="AN32" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO32" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP32" t="inlineStr"/>
+      <c r="AN32" t="inlineStr"/>
+      <c r="AO32" t="inlineStr"/>
+      <c r="AP32" t="inlineStr">
+        <is>
+          <t>ruins_shinier_entrance</t>
+        </is>
+      </c>
       <c r="AQ32" t="inlineStr"/>
-      <c r="AR32" t="inlineStr">
-        <is>
-          <t>ruins_shinier_entrance</t>
-        </is>
-      </c>
-      <c r="AS32" t="inlineStr"/>
+      <c r="AR32" t="inlineStr"/>
+      <c r="AS32" t="inlineStr">
+        <is>
+          <t>[{"id": "elf_antler", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT32" t="inlineStr"/>
-      <c r="AU32" t="inlineStr"/>
-      <c r="AV32" t="inlineStr">
-        <is>
-          <t>[{"id": "elf_antler", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW32" t="inlineStr"/>
-      <c r="AX32" t="inlineStr"/>
-      <c r="AY32" t="inlineStr"/>
-      <c r="AZ32" t="inlineStr"/>
     </row>
     <row r="33" ht="74.10000000000001" customHeight="1">
       <c r="A33" t="inlineStr">
@@ -6976,63 +6726,57 @@
         <v>5</v>
       </c>
       <c r="AE33" t="inlineStr"/>
-      <c r="AF33" t="inlineStr"/>
-      <c r="AG33" t="inlineStr"/>
-      <c r="AH33" t="inlineStr">
+      <c r="AF33" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH33" t="inlineStr"/>
       <c r="AI33" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ33" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK33" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL33" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM33" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN33" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO33" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP33" t="inlineStr"/>
+      <c r="AN33" t="inlineStr"/>
+      <c r="AO33" t="inlineStr"/>
+      <c r="AP33" t="inlineStr">
+        <is>
+          <t>Forest_Trail_Day</t>
+        </is>
+      </c>
       <c r="AQ33" t="inlineStr"/>
-      <c r="AR33" t="inlineStr">
-        <is>
-          <t>Forest_Trail_Day</t>
-        </is>
-      </c>
-      <c r="AS33" t="inlineStr"/>
+      <c r="AR33" t="inlineStr"/>
+      <c r="AS33" t="inlineStr">
+        <is>
+          <t>[{"id": "paw_bear", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT33" t="inlineStr"/>
-      <c r="AU33" t="inlineStr"/>
-      <c r="AV33" t="inlineStr">
-        <is>
-          <t>[{"id": "paw_bear", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW33" t="inlineStr"/>
-      <c r="AX33" t="inlineStr"/>
-      <c r="AY33" t="inlineStr"/>
-      <c r="AZ33" t="inlineStr"/>
     </row>
     <row r="34" ht="51.48" customHeight="1">
       <c r="A34" t="inlineStr">
@@ -7132,63 +6876,57 @@
         <v>5</v>
       </c>
       <c r="AE34" t="inlineStr"/>
-      <c r="AF34" t="inlineStr"/>
-      <c r="AG34" t="inlineStr"/>
-      <c r="AH34" t="inlineStr">
+      <c r="AF34" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG34" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH34" t="inlineStr"/>
       <c r="AI34" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ34" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK34" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL34" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM34" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN34" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO34" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP34" t="inlineStr"/>
+      <c r="AN34" t="inlineStr"/>
+      <c r="AO34" t="inlineStr"/>
+      <c r="AP34" t="inlineStr">
+        <is>
+          <t>Forest_Trail_Day</t>
+        </is>
+      </c>
       <c r="AQ34" t="inlineStr"/>
-      <c r="AR34" t="inlineStr">
-        <is>
-          <t>Forest_Trail_Day</t>
-        </is>
-      </c>
-      <c r="AS34" t="inlineStr"/>
+      <c r="AR34" t="inlineStr"/>
+      <c r="AS34" t="inlineStr">
+        <is>
+          <t>[{"id": "paw_bear", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT34" t="inlineStr"/>
-      <c r="AU34" t="inlineStr"/>
-      <c r="AV34" t="inlineStr">
-        <is>
-          <t>[{"id": "paw_bear", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW34" t="inlineStr"/>
-      <c r="AX34" t="inlineStr"/>
-      <c r="AY34" t="inlineStr"/>
-      <c r="AZ34" t="inlineStr"/>
     </row>
     <row r="35" ht="74.10000000000001" customHeight="1">
       <c r="A35" t="inlineStr">
@@ -7288,63 +7026,57 @@
         <v>5</v>
       </c>
       <c r="AE35" t="inlineStr"/>
-      <c r="AF35" t="inlineStr"/>
-      <c r="AG35" t="inlineStr"/>
-      <c r="AH35" t="inlineStr">
+      <c r="AF35" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG35" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH35" t="inlineStr"/>
       <c r="AI35" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ35" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK35" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL35" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM35" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN35" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO35" t="inlineStr">
-        <is>
           <t>right bottom</t>
         </is>
       </c>
-      <c r="AP35" t="inlineStr"/>
+      <c r="AN35" t="inlineStr"/>
+      <c r="AO35" t="inlineStr"/>
+      <c r="AP35" t="inlineStr">
+        <is>
+          <t>Forest_Cliff_Day</t>
+        </is>
+      </c>
       <c r="AQ35" t="inlineStr"/>
-      <c r="AR35" t="inlineStr">
-        <is>
-          <t>Forest_Cliff_Day</t>
-        </is>
-      </c>
-      <c r="AS35" t="inlineStr"/>
+      <c r="AR35" t="inlineStr"/>
+      <c r="AS35" t="inlineStr">
+        <is>
+          <t>[{"id": "antler_deer", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT35" t="inlineStr"/>
-      <c r="AU35" t="inlineStr"/>
-      <c r="AV35" t="inlineStr">
-        <is>
-          <t>[{"id": "antler_deer", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW35" t="inlineStr"/>
-      <c r="AX35" t="inlineStr"/>
-      <c r="AY35" t="inlineStr"/>
-      <c r="AZ35" t="inlineStr"/>
     </row>
     <row r="36" ht="42.12" customHeight="1">
       <c r="A36" t="inlineStr">
@@ -7444,63 +7176,57 @@
         <v>5</v>
       </c>
       <c r="AE36" t="inlineStr"/>
-      <c r="AF36" t="inlineStr"/>
-      <c r="AG36" t="inlineStr"/>
-      <c r="AH36" t="inlineStr">
+      <c r="AF36" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG36" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH36" t="inlineStr"/>
       <c r="AI36" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ36" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ36" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK36" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL36" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM36" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN36" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO36" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP36" t="inlineStr"/>
+      <c r="AN36" t="inlineStr"/>
+      <c r="AO36" t="inlineStr"/>
+      <c r="AP36" t="inlineStr">
+        <is>
+          <t>Forest_Cliff_Day</t>
+        </is>
+      </c>
       <c r="AQ36" t="inlineStr"/>
-      <c r="AR36" t="inlineStr">
-        <is>
-          <t>Forest_Cliff_Day</t>
-        </is>
-      </c>
-      <c r="AS36" t="inlineStr"/>
+      <c r="AR36" t="inlineStr"/>
+      <c r="AS36" t="inlineStr">
+        <is>
+          <t>[{"id": "antler_deer", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT36" t="inlineStr"/>
-      <c r="AU36" t="inlineStr"/>
-      <c r="AV36" t="inlineStr">
-        <is>
-          <t>[{"id": "antler_deer", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW36" t="inlineStr"/>
-      <c r="AX36" t="inlineStr"/>
-      <c r="AY36" t="inlineStr"/>
-      <c r="AZ36" t="inlineStr"/>
     </row>
     <row r="37" ht="74.88" customHeight="1">
       <c r="A37" t="inlineStr">
@@ -7600,63 +7326,57 @@
         <v>5</v>
       </c>
       <c r="AE37" t="inlineStr"/>
-      <c r="AF37" t="inlineStr"/>
-      <c r="AG37" t="inlineStr"/>
-      <c r="AH37" t="inlineStr">
+      <c r="AF37" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG37" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH37" t="inlineStr"/>
       <c r="AI37" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ37" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ37" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK37" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "bite"}, "wrong": {"type": "slash"}, "assault": {"type": "bite"}}</t>
         </is>
       </c>
       <c r="AL37" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM37" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "bite"}, "wrong": {"type": "slash"}, "assault": {"type": "bite"}}</t>
-        </is>
-      </c>
-      <c r="AN37" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO37" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP37" t="inlineStr"/>
+      <c r="AN37" t="inlineStr"/>
+      <c r="AO37" t="inlineStr"/>
+      <c r="AP37" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_Catacomb</t>
+        </is>
+      </c>
       <c r="AQ37" t="inlineStr"/>
-      <c r="AR37" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_Catacomb</t>
-        </is>
-      </c>
-      <c r="AS37" t="inlineStr"/>
+      <c r="AR37" t="inlineStr"/>
+      <c r="AS37" t="inlineStr">
+        <is>
+          <t>[{"id": "harm_bone", "n": 1, "p": 0.1}]</t>
+        </is>
+      </c>
       <c r="AT37" t="inlineStr"/>
-      <c r="AU37" t="inlineStr"/>
-      <c r="AV37" t="inlineStr">
-        <is>
-          <t>[{"id": "harm_bone", "n": 1, "p": 0.1}]</t>
-        </is>
-      </c>
-      <c r="AW37" t="inlineStr"/>
-      <c r="AX37" t="inlineStr"/>
-      <c r="AY37" t="inlineStr"/>
-      <c r="AZ37" t="inlineStr"/>
     </row>
     <row r="38" ht="74.88" customHeight="1">
       <c r="A38" t="inlineStr">
@@ -7756,63 +7476,57 @@
         <v>5</v>
       </c>
       <c r="AE38" t="inlineStr"/>
-      <c r="AF38" t="inlineStr"/>
-      <c r="AG38" t="inlineStr"/>
-      <c r="AH38" t="inlineStr">
+      <c r="AF38" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH38" t="inlineStr"/>
       <c r="AI38" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ38" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ38" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 16]</t>
+        </is>
+      </c>
       <c r="AK38" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt", "count": 2}}</t>
         </is>
       </c>
       <c r="AL38" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 16]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM38" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt", "count": 2}}</t>
-        </is>
-      </c>
-      <c r="AN38" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO38" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP38" t="inlineStr"/>
+      <c r="AN38" t="inlineStr"/>
+      <c r="AO38" t="inlineStr"/>
+      <c r="AP38" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_Colossus</t>
+        </is>
+      </c>
       <c r="AQ38" t="inlineStr"/>
-      <c r="AR38" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_Colossus</t>
-        </is>
-      </c>
-      <c r="AS38" t="inlineStr"/>
+      <c r="AR38" t="inlineStr"/>
+      <c r="AS38" t="inlineStr">
+        <is>
+          <t>[{"id": "bell_shard", "n": 1, "p": 0.1}]</t>
+        </is>
+      </c>
       <c r="AT38" t="inlineStr"/>
-      <c r="AU38" t="inlineStr"/>
-      <c r="AV38" t="inlineStr">
-        <is>
-          <t>[{"id": "bell_shard", "n": 1, "p": 0.1}]</t>
-        </is>
-      </c>
-      <c r="AW38" t="inlineStr"/>
-      <c r="AX38" t="inlineStr"/>
-      <c r="AY38" t="inlineStr"/>
-      <c r="AZ38" t="inlineStr"/>
     </row>
     <row r="39" ht="74.88" customHeight="1">
       <c r="A39" t="inlineStr">
@@ -7912,63 +7626,57 @@
         <v>5</v>
       </c>
       <c r="AE39" t="inlineStr"/>
-      <c r="AF39" t="inlineStr"/>
-      <c r="AG39" t="inlineStr"/>
-      <c r="AH39" t="inlineStr">
+      <c r="AF39" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG39" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH39" t="inlineStr"/>
       <c r="AI39" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ39" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ39" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK39" t="inlineStr">
         <is>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
+        </is>
+      </c>
+      <c r="AL39" t="inlineStr">
+        <is>
+          <t>contain</t>
+        </is>
+      </c>
+      <c r="AM39" t="inlineStr">
+        <is>
+          <t>center bottom</t>
+        </is>
+      </c>
+      <c r="AN39" t="inlineStr"/>
+      <c r="AO39" t="inlineStr"/>
+      <c r="AP39" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_Hollow</t>
+        </is>
+      </c>
+      <c r="AQ39" t="inlineStr"/>
+      <c r="AR39" t="inlineStr"/>
+      <c r="AS39" t="inlineStr">
+        <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AL39" t="inlineStr">
-        <is>
-          <t>[9, 9, 9, 9, 9]</t>
-        </is>
-      </c>
-      <c r="AM39" t="inlineStr">
-        <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN39" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO39" t="inlineStr">
-        <is>
-          <t>center bottom</t>
-        </is>
-      </c>
-      <c r="AP39" t="inlineStr"/>
-      <c r="AQ39" t="inlineStr"/>
-      <c r="AR39" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_Hollow</t>
-        </is>
-      </c>
-      <c r="AS39" t="inlineStr"/>
       <c r="AT39" t="inlineStr"/>
-      <c r="AU39" t="inlineStr"/>
-      <c r="AV39" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AW39" t="inlineStr"/>
-      <c r="AX39" t="inlineStr"/>
-      <c r="AY39" t="inlineStr"/>
-      <c r="AZ39" t="inlineStr"/>
     </row>
     <row r="40" ht="74.88" customHeight="1">
       <c r="A40" t="inlineStr">
@@ -8068,63 +7776,57 @@
         <v>5</v>
       </c>
       <c r="AE40" t="inlineStr"/>
-      <c r="AF40" t="inlineStr"/>
-      <c r="AG40" t="inlineStr"/>
-      <c r="AH40" t="inlineStr">
+      <c r="AF40" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG40" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH40" t="inlineStr"/>
       <c r="AI40" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ40" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ40" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK40" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "claw", "count": 1, "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL40" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM40" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "claw", "count": 1, "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN40" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO40" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP40" t="inlineStr"/>
+      <c r="AN40" t="inlineStr"/>
+      <c r="AO40" t="inlineStr"/>
+      <c r="AP40" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_Prison</t>
+        </is>
+      </c>
       <c r="AQ40" t="inlineStr"/>
-      <c r="AR40" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_Prison</t>
-        </is>
-      </c>
-      <c r="AS40" t="inlineStr"/>
+      <c r="AR40" t="inlineStr"/>
+      <c r="AS40" t="inlineStr">
+        <is>
+          <t>[{"id": "harm_claw", "n": 1, "p": 0.1}]</t>
+        </is>
+      </c>
       <c r="AT40" t="inlineStr"/>
-      <c r="AU40" t="inlineStr"/>
-      <c r="AV40" t="inlineStr">
-        <is>
-          <t>[{"id": "harm_claw", "n": 1, "p": 0.1}]</t>
-        </is>
-      </c>
-      <c r="AW40" t="inlineStr"/>
-      <c r="AX40" t="inlineStr"/>
-      <c r="AY40" t="inlineStr"/>
-      <c r="AZ40" t="inlineStr"/>
     </row>
     <row r="41" ht="74.10000000000001" customHeight="1">
       <c r="A41" t="inlineStr">
@@ -8224,63 +7926,57 @@
         <v>5</v>
       </c>
       <c r="AE41" t="inlineStr"/>
-      <c r="AF41" t="inlineStr"/>
-      <c r="AG41" t="inlineStr"/>
-      <c r="AH41" t="inlineStr">
+      <c r="AF41" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG41" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH41" t="inlineStr"/>
       <c r="AI41" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ41" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ41" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK41" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL41" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM41" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN41" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO41" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP41" t="inlineStr"/>
+      <c r="AN41" t="inlineStr"/>
+      <c r="AO41" t="inlineStr"/>
+      <c r="AP41" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ41" t="inlineStr"/>
-      <c r="AR41" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
-      <c r="AS41" t="inlineStr"/>
+      <c r="AR41" t="inlineStr"/>
+      <c r="AS41" t="inlineStr">
+        <is>
+          <t>[{"id": "bell_shard", "n": 1, "p": 0.1}]</t>
+        </is>
+      </c>
       <c r="AT41" t="inlineStr"/>
-      <c r="AU41" t="inlineStr"/>
-      <c r="AV41" t="inlineStr">
-        <is>
-          <t>[{"id": "bell_shard", "n": 1, "p": 0.1}]</t>
-        </is>
-      </c>
-      <c r="AW41" t="inlineStr"/>
-      <c r="AX41" t="inlineStr"/>
-      <c r="AY41" t="inlineStr"/>
-      <c r="AZ41" t="inlineStr"/>
     </row>
     <row r="42" ht="74.88" customHeight="1">
       <c r="A42" t="inlineStr">
@@ -8380,63 +8076,57 @@
         <v>5</v>
       </c>
       <c r="AE42" t="inlineStr"/>
-      <c r="AF42" t="inlineStr"/>
-      <c r="AG42" t="inlineStr"/>
-      <c r="AH42" t="inlineStr">
+      <c r="AF42" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG42" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH42" t="inlineStr"/>
       <c r="AI42" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ42" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ42" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK42" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL42" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM42" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN42" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO42" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP42" t="inlineStr"/>
+      <c r="AN42" t="inlineStr"/>
+      <c r="AO42" t="inlineStr"/>
+      <c r="AP42" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_Prison</t>
+        </is>
+      </c>
       <c r="AQ42" t="inlineStr"/>
-      <c r="AR42" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_Prison</t>
-        </is>
-      </c>
-      <c r="AS42" t="inlineStr"/>
+      <c r="AR42" t="inlineStr"/>
+      <c r="AS42" t="inlineStr">
+        <is>
+          <t>[{"id": "saint_claw", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT42" t="inlineStr"/>
-      <c r="AU42" t="inlineStr"/>
-      <c r="AV42" t="inlineStr">
-        <is>
-          <t>[{"id": "saint_claw", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW42" t="inlineStr"/>
-      <c r="AX42" t="inlineStr"/>
-      <c r="AY42" t="inlineStr"/>
-      <c r="AZ42" t="inlineStr"/>
     </row>
     <row r="43" ht="74.88" customHeight="1">
       <c r="A43" t="inlineStr">
@@ -8536,63 +8226,57 @@
         <v>5</v>
       </c>
       <c r="AE43" t="inlineStr"/>
-      <c r="AF43" t="inlineStr"/>
-      <c r="AG43" t="inlineStr"/>
-      <c r="AH43" t="inlineStr">
+      <c r="AF43" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG43" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH43" t="inlineStr"/>
       <c r="AI43" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ43" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ43" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 16]</t>
+        </is>
+      </c>
       <c r="AK43" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "slash"}, "wrong": {"type": "slash"}, "assault": {"type": "slash", "count": 2}}</t>
         </is>
       </c>
       <c r="AL43" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 16]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM43" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "slash"}, "wrong": {"type": "slash"}, "assault": {"type": "slash", "count": 2}}</t>
-        </is>
-      </c>
-      <c r="AN43" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO43" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP43" t="inlineStr"/>
+      <c r="AN43" t="inlineStr"/>
+      <c r="AO43" t="inlineStr"/>
+      <c r="AP43" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_DarkBridge</t>
+        </is>
+      </c>
       <c r="AQ43" t="inlineStr"/>
-      <c r="AR43" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_DarkBridge</t>
-        </is>
-      </c>
-      <c r="AS43" t="inlineStr"/>
+      <c r="AR43" t="inlineStr"/>
+      <c r="AS43" t="inlineStr">
+        <is>
+          <t>[{"id": "saint_fang", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT43" t="inlineStr"/>
-      <c r="AU43" t="inlineStr"/>
-      <c r="AV43" t="inlineStr">
-        <is>
-          <t>[{"id": "saint_fang", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW43" t="inlineStr"/>
-      <c r="AX43" t="inlineStr"/>
-      <c r="AY43" t="inlineStr"/>
-      <c r="AZ43" t="inlineStr"/>
     </row>
     <row r="44" ht="74.88" customHeight="1">
       <c r="A44" t="inlineStr">
@@ -8692,63 +8376,57 @@
         <v>5</v>
       </c>
       <c r="AE44" t="inlineStr"/>
-      <c r="AF44" t="inlineStr"/>
-      <c r="AG44" t="inlineStr"/>
-      <c r="AH44" t="inlineStr">
+      <c r="AF44" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG44" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH44" t="inlineStr"/>
       <c r="AI44" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ44" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ44" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 16]</t>
+        </is>
+      </c>
       <c r="AK44" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt", "count": 2}}</t>
         </is>
       </c>
       <c r="AL44" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 16]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM44" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt", "count": 2}}</t>
-        </is>
-      </c>
-      <c r="AN44" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO44" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP44" t="inlineStr"/>
+      <c r="AN44" t="inlineStr"/>
+      <c r="AO44" t="inlineStr"/>
+      <c r="AP44" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_CorridorA</t>
+        </is>
+      </c>
       <c r="AQ44" t="inlineStr"/>
-      <c r="AR44" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_CorridorA</t>
-        </is>
-      </c>
-      <c r="AS44" t="inlineStr"/>
+      <c r="AR44" t="inlineStr"/>
+      <c r="AS44" t="inlineStr">
+        <is>
+          <t>[{"id": "saint_bone_big", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT44" t="inlineStr"/>
-      <c r="AU44" t="inlineStr"/>
-      <c r="AV44" t="inlineStr">
-        <is>
-          <t>[{"id": "saint_bone_big", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW44" t="inlineStr"/>
-      <c r="AX44" t="inlineStr"/>
-      <c r="AY44" t="inlineStr"/>
-      <c r="AZ44" t="inlineStr"/>
     </row>
     <row r="45" ht="74.88" customHeight="1">
       <c r="A45" t="inlineStr">
@@ -8848,63 +8526,57 @@
         <v>5</v>
       </c>
       <c r="AE45" t="inlineStr"/>
-      <c r="AF45" t="inlineStr"/>
-      <c r="AG45" t="inlineStr"/>
-      <c r="AH45" t="inlineStr">
+      <c r="AF45" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH45" t="inlineStr"/>
       <c r="AI45" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ45" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ45" t="inlineStr">
+        <is>
+          <t>[9, 9, 16, 9, 16]</t>
+        </is>
+      </c>
       <c r="AK45" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
         </is>
       </c>
       <c r="AL45" t="inlineStr">
         <is>
-          <t>[9, 9, 16, 9, 16]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM45" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blunt"}, "wrong": {"type": "slash"}, "assault": {"type": "claw", "count": 3, "angle": "random"}}</t>
-        </is>
-      </c>
-      <c r="AN45" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO45" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP45" t="inlineStr"/>
+      <c r="AN45" t="inlineStr"/>
+      <c r="AO45" t="inlineStr"/>
+      <c r="AP45" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_DeepAltar</t>
+        </is>
+      </c>
       <c r="AQ45" t="inlineStr"/>
-      <c r="AR45" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_DeepAltar</t>
-        </is>
-      </c>
-      <c r="AS45" t="inlineStr"/>
+      <c r="AR45" t="inlineStr"/>
+      <c r="AS45" t="inlineStr">
+        <is>
+          <t>[{"id": "saint_bone", "n": 1}]</t>
+        </is>
+      </c>
       <c r="AT45" t="inlineStr"/>
-      <c r="AU45" t="inlineStr"/>
-      <c r="AV45" t="inlineStr">
-        <is>
-          <t>[{"id": "saint_bone", "n": 1}]</t>
-        </is>
-      </c>
-      <c r="AW45" t="inlineStr"/>
-      <c r="AX45" t="inlineStr"/>
-      <c r="AY45" t="inlineStr"/>
-      <c r="AZ45" t="inlineStr"/>
     </row>
     <row r="46" ht="74.88" customHeight="1">
       <c r="A46" t="inlineStr">
@@ -9004,59 +8676,53 @@
         <v>5</v>
       </c>
       <c r="AE46" t="inlineStr"/>
-      <c r="AF46" t="inlineStr"/>
-      <c r="AG46" t="inlineStr"/>
-      <c r="AH46" t="inlineStr">
+      <c r="AF46" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH46" t="inlineStr"/>
       <c r="AI46" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ46" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ46" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK46" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL46" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM46" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN46" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO46" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP46" t="inlineStr"/>
+      <c r="AN46" t="inlineStr"/>
+      <c r="AO46" t="inlineStr"/>
+      <c r="AP46" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ46" t="inlineStr"/>
-      <c r="AR46" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
+      <c r="AR46" t="inlineStr"/>
       <c r="AS46" t="inlineStr"/>
       <c r="AT46" t="inlineStr"/>
-      <c r="AU46" t="inlineStr"/>
-      <c r="AV46" t="inlineStr"/>
-      <c r="AW46" t="inlineStr"/>
-      <c r="AX46" t="inlineStr"/>
-      <c r="AY46" t="inlineStr"/>
-      <c r="AZ46" t="inlineStr"/>
     </row>
     <row r="47" ht="74.88" customHeight="1">
       <c r="A47" t="inlineStr">
@@ -9156,59 +8822,53 @@
         <v>5</v>
       </c>
       <c r="AE47" t="inlineStr"/>
-      <c r="AF47" t="inlineStr"/>
-      <c r="AG47" t="inlineStr"/>
-      <c r="AH47" t="inlineStr">
+      <c r="AF47" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG47" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH47" t="inlineStr"/>
       <c r="AI47" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ47" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ47" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK47" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL47" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM47" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN47" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO47" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP47" t="inlineStr"/>
+      <c r="AN47" t="inlineStr"/>
+      <c r="AO47" t="inlineStr"/>
+      <c r="AP47" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ47" t="inlineStr"/>
-      <c r="AR47" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
+      <c r="AR47" t="inlineStr"/>
       <c r="AS47" t="inlineStr"/>
       <c r="AT47" t="inlineStr"/>
-      <c r="AU47" t="inlineStr"/>
-      <c r="AV47" t="inlineStr"/>
-      <c r="AW47" t="inlineStr"/>
-      <c r="AX47" t="inlineStr"/>
-      <c r="AY47" t="inlineStr"/>
-      <c r="AZ47" t="inlineStr"/>
     </row>
     <row r="48" ht="74.88" customHeight="1">
       <c r="A48" t="inlineStr">
@@ -9308,59 +8968,53 @@
         <v>5</v>
       </c>
       <c r="AE48" t="inlineStr"/>
-      <c r="AF48" t="inlineStr"/>
-      <c r="AG48" t="inlineStr"/>
-      <c r="AH48" t="inlineStr">
+      <c r="AF48" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG48" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH48" t="inlineStr"/>
       <c r="AI48" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ48" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ48" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK48" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL48" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM48" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN48" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO48" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP48" t="inlineStr"/>
+      <c r="AN48" t="inlineStr"/>
+      <c r="AO48" t="inlineStr"/>
+      <c r="AP48" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ48" t="inlineStr"/>
-      <c r="AR48" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
+      <c r="AR48" t="inlineStr"/>
       <c r="AS48" t="inlineStr"/>
       <c r="AT48" t="inlineStr"/>
-      <c r="AU48" t="inlineStr"/>
-      <c r="AV48" t="inlineStr"/>
-      <c r="AW48" t="inlineStr"/>
-      <c r="AX48" t="inlineStr"/>
-      <c r="AY48" t="inlineStr"/>
-      <c r="AZ48" t="inlineStr"/>
     </row>
     <row r="49" ht="74.88" customHeight="1">
       <c r="A49" t="inlineStr">
@@ -9460,59 +9114,53 @@
         <v>5</v>
       </c>
       <c r="AE49" t="inlineStr"/>
-      <c r="AF49" t="inlineStr"/>
-      <c r="AG49" t="inlineStr"/>
-      <c r="AH49" t="inlineStr">
+      <c r="AF49" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG49" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH49" t="inlineStr"/>
       <c r="AI49" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ49" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ49" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK49" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL49" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM49" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN49" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO49" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP49" t="inlineStr"/>
+      <c r="AN49" t="inlineStr"/>
+      <c r="AO49" t="inlineStr"/>
+      <c r="AP49" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ49" t="inlineStr"/>
-      <c r="AR49" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
+      <c r="AR49" t="inlineStr"/>
       <c r="AS49" t="inlineStr"/>
       <c r="AT49" t="inlineStr"/>
-      <c r="AU49" t="inlineStr"/>
-      <c r="AV49" t="inlineStr"/>
-      <c r="AW49" t="inlineStr"/>
-      <c r="AX49" t="inlineStr"/>
-      <c r="AY49" t="inlineStr"/>
-      <c r="AZ49" t="inlineStr"/>
     </row>
     <row r="50" ht="74.88" customHeight="1">
       <c r="A50" t="inlineStr">
@@ -9612,59 +9260,53 @@
         <v>5</v>
       </c>
       <c r="AE50" t="inlineStr"/>
-      <c r="AF50" t="inlineStr"/>
-      <c r="AG50" t="inlineStr"/>
-      <c r="AH50" t="inlineStr">
+      <c r="AF50" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG50" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH50" t="inlineStr"/>
       <c r="AI50" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ50" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ50" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK50" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL50" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM50" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN50" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO50" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP50" t="inlineStr"/>
+      <c r="AN50" t="inlineStr"/>
+      <c r="AO50" t="inlineStr"/>
+      <c r="AP50" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ50" t="inlineStr"/>
-      <c r="AR50" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
+      <c r="AR50" t="inlineStr"/>
       <c r="AS50" t="inlineStr"/>
       <c r="AT50" t="inlineStr"/>
-      <c r="AU50" t="inlineStr"/>
-      <c r="AV50" t="inlineStr"/>
-      <c r="AW50" t="inlineStr"/>
-      <c r="AX50" t="inlineStr"/>
-      <c r="AY50" t="inlineStr"/>
-      <c r="AZ50" t="inlineStr"/>
     </row>
     <row r="51" ht="74.88" customHeight="1">
       <c r="A51" t="inlineStr">
@@ -9764,59 +9406,53 @@
         <v>5</v>
       </c>
       <c r="AE51" t="inlineStr"/>
-      <c r="AF51" t="inlineStr"/>
-      <c r="AG51" t="inlineStr"/>
-      <c r="AH51" t="inlineStr">
+      <c r="AF51" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG51" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH51" t="inlineStr"/>
       <c r="AI51" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ51" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ51" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK51" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL51" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM51" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN51" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO51" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP51" t="inlineStr"/>
+      <c r="AN51" t="inlineStr"/>
+      <c r="AO51" t="inlineStr"/>
+      <c r="AP51" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ51" t="inlineStr"/>
-      <c r="AR51" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
+      <c r="AR51" t="inlineStr"/>
       <c r="AS51" t="inlineStr"/>
       <c r="AT51" t="inlineStr"/>
-      <c r="AU51" t="inlineStr"/>
-      <c r="AV51" t="inlineStr"/>
-      <c r="AW51" t="inlineStr"/>
-      <c r="AX51" t="inlineStr"/>
-      <c r="AY51" t="inlineStr"/>
-      <c r="AZ51" t="inlineStr"/>
     </row>
     <row r="52" ht="74.88" customHeight="1">
       <c r="A52" t="inlineStr">
@@ -9916,59 +9552,53 @@
         <v>5</v>
       </c>
       <c r="AE52" t="inlineStr"/>
-      <c r="AF52" t="inlineStr"/>
-      <c r="AG52" t="inlineStr"/>
-      <c r="AH52" t="inlineStr">
+      <c r="AF52" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH52" t="inlineStr"/>
       <c r="AI52" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ52" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ52" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK52" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL52" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM52" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN52" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO52" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP52" t="inlineStr"/>
+      <c r="AN52" t="inlineStr"/>
+      <c r="AO52" t="inlineStr"/>
+      <c r="AP52" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ52" t="inlineStr"/>
-      <c r="AR52" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
+      <c r="AR52" t="inlineStr"/>
       <c r="AS52" t="inlineStr"/>
       <c r="AT52" t="inlineStr"/>
-      <c r="AU52" t="inlineStr"/>
-      <c r="AV52" t="inlineStr"/>
-      <c r="AW52" t="inlineStr"/>
-      <c r="AX52" t="inlineStr"/>
-      <c r="AY52" t="inlineStr"/>
-      <c r="AZ52" t="inlineStr"/>
     </row>
     <row r="53" ht="74.88" customHeight="1">
       <c r="A53" t="inlineStr">
@@ -10068,59 +9698,53 @@
         <v>5</v>
       </c>
       <c r="AE53" t="inlineStr"/>
-      <c r="AF53" t="inlineStr"/>
-      <c r="AG53" t="inlineStr"/>
-      <c r="AH53" t="inlineStr">
+      <c r="AF53" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG53" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH53" t="inlineStr"/>
       <c r="AI53" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ53" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ53" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK53" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL53" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM53" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN53" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO53" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP53" t="inlineStr"/>
+      <c r="AN53" t="inlineStr"/>
+      <c r="AO53" t="inlineStr"/>
+      <c r="AP53" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ53" t="inlineStr"/>
-      <c r="AR53" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
+      <c r="AR53" t="inlineStr"/>
       <c r="AS53" t="inlineStr"/>
       <c r="AT53" t="inlineStr"/>
-      <c r="AU53" t="inlineStr"/>
-      <c r="AV53" t="inlineStr"/>
-      <c r="AW53" t="inlineStr"/>
-      <c r="AX53" t="inlineStr"/>
-      <c r="AY53" t="inlineStr"/>
-      <c r="AZ53" t="inlineStr"/>
     </row>
     <row r="54" ht="74.88" customHeight="1">
       <c r="A54" t="inlineStr">
@@ -10220,59 +9844,53 @@
         <v>5</v>
       </c>
       <c r="AE54" t="inlineStr"/>
-      <c r="AF54" t="inlineStr"/>
-      <c r="AG54" t="inlineStr"/>
-      <c r="AH54" t="inlineStr">
+      <c r="AF54" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG54" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH54" t="inlineStr"/>
       <c r="AI54" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ54" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ54" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK54" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL54" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM54" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN54" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO54" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP54" t="inlineStr"/>
+      <c r="AN54" t="inlineStr"/>
+      <c r="AO54" t="inlineStr"/>
+      <c r="AP54" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ54" t="inlineStr"/>
-      <c r="AR54" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
+      <c r="AR54" t="inlineStr"/>
       <c r="AS54" t="inlineStr"/>
       <c r="AT54" t="inlineStr"/>
-      <c r="AU54" t="inlineStr"/>
-      <c r="AV54" t="inlineStr"/>
-      <c r="AW54" t="inlineStr"/>
-      <c r="AX54" t="inlineStr"/>
-      <c r="AY54" t="inlineStr"/>
-      <c r="AZ54" t="inlineStr"/>
     </row>
     <row r="55" ht="74.88" customHeight="1">
       <c r="A55" t="inlineStr">
@@ -10372,59 +9990,53 @@
         <v>5</v>
       </c>
       <c r="AE55" t="inlineStr"/>
-      <c r="AF55" t="inlineStr"/>
-      <c r="AG55" t="inlineStr"/>
-      <c r="AH55" t="inlineStr">
+      <c r="AF55" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="AG55" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH55" t="inlineStr"/>
       <c r="AI55" t="inlineStr">
         <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="AJ55" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AJ55" t="inlineStr">
+        <is>
+          <t>[9, 9, 9, 9, 9]</t>
+        </is>
+      </c>
       <c r="AK55" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
         </is>
       </c>
       <c r="AL55" t="inlineStr">
         <is>
-          <t>[9, 9, 9, 9, 9]</t>
+          <t>contain</t>
         </is>
       </c>
       <c r="AM55" t="inlineStr">
         <is>
-          <t>{"delay": {"type": "blood", "angle": "random"}, "wrong": {"type": "slash"}, "assault": {"type": "blunt"}}</t>
-        </is>
-      </c>
-      <c r="AN55" t="inlineStr">
-        <is>
-          <t>contain</t>
-        </is>
-      </c>
-      <c r="AO55" t="inlineStr">
-        <is>
           <t>center bottom</t>
         </is>
       </c>
-      <c r="AP55" t="inlineStr"/>
+      <c r="AN55" t="inlineStr"/>
+      <c r="AO55" t="inlineStr"/>
+      <c r="AP55" t="inlineStr">
+        <is>
+          <t>Ruins_shinier_MossChamber</t>
+        </is>
+      </c>
       <c r="AQ55" t="inlineStr"/>
-      <c r="AR55" t="inlineStr">
-        <is>
-          <t>Ruins_shinier_MossChamber</t>
-        </is>
-      </c>
+      <c r="AR55" t="inlineStr"/>
       <c r="AS55" t="inlineStr"/>
       <c r="AT55" t="inlineStr"/>
-      <c r="AU55" t="inlineStr"/>
-      <c r="AV55" t="inlineStr"/>
-      <c r="AW55" t="inlineStr"/>
-      <c r="AX55" t="inlineStr"/>
-      <c r="AY55" t="inlineStr"/>
-      <c r="AZ55" t="inlineStr"/>
     </row>
     <row r="56" ht="74.88" customHeight="1">
       <c r="A56" t="inlineStr"/>
@@ -10477,12 +10089,6 @@
       <c r="AR56" t="inlineStr"/>
       <c r="AS56" t="inlineStr"/>
       <c r="AT56" t="inlineStr"/>
-      <c r="AU56" t="inlineStr"/>
-      <c r="AV56" t="inlineStr"/>
-      <c r="AW56" t="inlineStr"/>
-      <c r="AX56" t="inlineStr"/>
-      <c r="AY56" t="inlineStr"/>
-      <c r="AZ56" t="inlineStr"/>
     </row>
     <row r="57" ht="74.88" customHeight="1">
       <c r="A57" t="inlineStr"/>
@@ -10535,12 +10141,6 @@
       <c r="AR57" t="inlineStr"/>
       <c r="AS57" t="inlineStr"/>
       <c r="AT57" t="inlineStr"/>
-      <c r="AU57" t="inlineStr"/>
-      <c r="AV57" t="inlineStr"/>
-      <c r="AW57" t="inlineStr"/>
-      <c r="AX57" t="inlineStr"/>
-      <c r="AY57" t="inlineStr"/>
-      <c r="AZ57" t="inlineStr"/>
     </row>
     <row r="58" ht="74.88" customHeight="1">
       <c r="A58" t="inlineStr"/>
@@ -10593,12 +10193,6 @@
       <c r="AR58" t="inlineStr"/>
       <c r="AS58" t="inlineStr"/>
       <c r="AT58" t="inlineStr"/>
-      <c r="AU58" t="inlineStr"/>
-      <c r="AV58" t="inlineStr"/>
-      <c r="AW58" t="inlineStr"/>
-      <c r="AX58" t="inlineStr"/>
-      <c r="AY58" t="inlineStr"/>
-      <c r="AZ58" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10623,7 +10217,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>127aa6497160cada366228d750732ac2cd3616e8fee2b2f1eec4e00d2d18eaff</t>
+          <t>48fce4d0cc9b8e0e46596adbd555eb6ea414f7e878f93e135e2d78e7f9cf6ce1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(enemy): entranceVo 與 landSe 併成一格 entranceSe ver -948
Ray：「entranceVo 跟 landSe 應該是同一時間發生，併為一格」

卡上只剩 entranceSe，**播的時機由這隻怪自己決定**：
  · 有降臨的（ENTRANCE_KINDS：禍魘／聖徒／船）→ 著地那一刻
  · 沒有降臨的（human…）                      → 立繪出現那一刻
對玩家而言那就是同一件事（「牠登場了」），資料上不該是兩格。

⚠ 走哪一軌是**算出來的**（playEntranceSe 一支，鐵律 7/8）：路徑落在 /vo/ 就走
  playVoice（過 voiceChain、吃 VO 分層音量），否則走 play（SE）。判**路徑**不判
  鑰匙前綴 —— 鑰匙的命名不是每個都守規約（sfx_saint 就不是 se_ 開頭），
  而路徑是檔案實際住哪一層，那才是「它是不是語音」的事實。

⚠⚠ 合併時踩到一個會沉默吃掉資料的坑：man_sorana **兩個欄位都有**
  （entranceVo:'vo_sorana_pack2' 與 landSe:null），改名之後同一個物件裡出現兩個
  entranceSe，**後面那個 null 蓋掉前面** → 她的登場語音直接消失，而且不會報錯。
  已刪掉多餘那一行，並加一道全欄位重名自檢（現在 0 張卡重名）。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/enemies.xlsx
+++ b/tools/enemies.xlsx
@@ -1855,7 +1855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT58"/>
+  <dimension ref="A1:AS58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1897,13 +1897,12 @@
     <col width="46" customWidth="1" min="37" max="37"/>
     <col width="10" customWidth="1" min="38" max="38"/>
     <col width="15" customWidth="1" min="39" max="39"/>
-    <col width="17" customWidth="1" min="40" max="40"/>
-    <col width="9" customWidth="1" min="41" max="41"/>
-    <col width="27" customWidth="1" min="42" max="42"/>
-    <col width="11" customWidth="1" min="43" max="43"/>
-    <col width="21" customWidth="1" min="44" max="44"/>
-    <col width="46" customWidth="1" min="45" max="45"/>
-    <col width="25" customWidth="1" min="46" max="46"/>
+    <col width="9" customWidth="1" min="40" max="40"/>
+    <col width="27" customWidth="1" min="41" max="41"/>
+    <col width="11" customWidth="1" min="42" max="42"/>
+    <col width="21" customWidth="1" min="43" max="43"/>
+    <col width="46" customWidth="1" min="44" max="44"/>
+    <col width="25" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2074,7 +2073,7 @@
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>landSe</t>
+          <t>entranceSe</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
@@ -2104,35 +2103,30 @@
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>entranceVo</t>
+          <t>noStack</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>noStack</t>
+          <t>bg</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
         <is>
-          <t>bg</t>
+          <t>boardLoop</t>
         </is>
       </c>
       <c r="AQ1" s="1" t="inlineStr">
         <is>
-          <t>boardLoop</t>
+          <t>wrongPenalty.damage</t>
         </is>
       </c>
       <c r="AR1" s="1" t="inlineStr">
         <is>
-          <t>wrongPenalty.damage</t>
+          <t>loot</t>
         </is>
       </c>
       <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>loot</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>money</t>
         </is>
@@ -2270,7 +2264,6 @@
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
     </row>
     <row r="3" ht="49.92" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -2404,7 +2397,6 @@
       <c r="AQ3" t="inlineStr"/>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
     </row>
     <row r="4" ht="62.40000000000001" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -2536,7 +2528,6 @@
       <c r="AQ4" t="inlineStr"/>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr"/>
     </row>
     <row r="5" ht="62.40000000000001" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -2668,7 +2659,6 @@
       <c r="AQ5" t="inlineStr"/>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="inlineStr"/>
-      <c r="AT5" t="inlineStr"/>
     </row>
     <row r="6" ht="52.26000000000001" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -2808,7 +2798,6 @@
       <c r="AQ6" t="inlineStr"/>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="inlineStr"/>
-      <c r="AT6" t="inlineStr"/>
     </row>
     <row r="7" ht="74.88" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -2920,7 +2909,11 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="AH7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>vo_sorana_pack2</t>
+        </is>
+      </c>
       <c r="AI7" t="inlineStr">
         <is>
           <t>[]</t>
@@ -2942,19 +2935,14 @@
           <t>50% 30%</t>
         </is>
       </c>
-      <c r="AN7" t="inlineStr">
-        <is>
-          <t>vo_sorana_pack2</t>
-        </is>
-      </c>
-      <c r="AO7" t="b">
-        <v>1</v>
-      </c>
+      <c r="AN7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO7" t="inlineStr"/>
       <c r="AP7" t="inlineStr"/>
       <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="inlineStr"/>
-      <c r="AT7" t="inlineStr"/>
     </row>
     <row r="8" ht="74.88" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -3094,7 +3082,6 @@
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="inlineStr"/>
-      <c r="AT8" t="inlineStr"/>
     </row>
     <row r="9" ht="70.98" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -3224,7 +3211,6 @@
       <c r="AQ9" t="inlineStr"/>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="inlineStr"/>
-      <c r="AT9" t="inlineStr"/>
     </row>
     <row r="10" ht="62.40000000000001" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -3356,7 +3342,6 @@
       <c r="AQ10" t="inlineStr"/>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
-      <c r="AT10" t="inlineStr"/>
     </row>
     <row r="11" ht="74.10000000000001" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -3493,16 +3478,15 @@
         </is>
       </c>
       <c r="AN11" t="inlineStr"/>
-      <c r="AO11" t="inlineStr"/>
-      <c r="AP11" t="inlineStr">
+      <c r="AO11" t="inlineStr">
         <is>
           <t>Northport_church_BF</t>
         </is>
       </c>
+      <c r="AP11" t="inlineStr"/>
       <c r="AQ11" t="inlineStr"/>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr"/>
-      <c r="AT11" t="inlineStr"/>
     </row>
     <row r="12" ht="74.88" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -3639,16 +3623,15 @@
         </is>
       </c>
       <c r="AN12" t="inlineStr"/>
-      <c r="AO12" t="inlineStr"/>
-      <c r="AP12" t="inlineStr">
+      <c r="AO12" t="inlineStr">
         <is>
           <t>Northport_church_BF</t>
         </is>
       </c>
+      <c r="AP12" t="inlineStr"/>
       <c r="AQ12" t="inlineStr"/>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
-      <c r="AT12" t="inlineStr"/>
     </row>
     <row r="13" ht="74.88" customHeight="1">
       <c r="A13" t="inlineStr">
@@ -3785,16 +3768,15 @@
         </is>
       </c>
       <c r="AN13" t="inlineStr"/>
-      <c r="AO13" t="inlineStr"/>
-      <c r="AP13" t="inlineStr">
+      <c r="AO13" t="inlineStr">
         <is>
           <t>Northport_church_BF</t>
         </is>
       </c>
+      <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="inlineStr"/>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
-      <c r="AT13" t="inlineStr"/>
     </row>
     <row r="14" ht="74.10000000000001" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -3931,16 +3913,15 @@
         </is>
       </c>
       <c r="AN14" t="inlineStr"/>
-      <c r="AO14" t="inlineStr"/>
-      <c r="AP14" t="inlineStr">
+      <c r="AO14" t="inlineStr">
         <is>
           <t>Northport_church_BF</t>
         </is>
       </c>
+      <c r="AP14" t="inlineStr"/>
       <c r="AQ14" t="inlineStr"/>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
-      <c r="AT14" t="inlineStr"/>
     </row>
     <row r="15" ht="74.88" customHeight="1">
       <c r="A15" t="inlineStr">
@@ -4077,16 +4058,15 @@
         </is>
       </c>
       <c r="AN15" t="inlineStr"/>
-      <c r="AO15" t="inlineStr"/>
-      <c r="AP15" t="inlineStr">
+      <c r="AO15" t="inlineStr">
         <is>
           <t>Northport_church_BF</t>
         </is>
       </c>
+      <c r="AP15" t="inlineStr"/>
       <c r="AQ15" t="inlineStr"/>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="inlineStr"/>
-      <c r="AT15" t="inlineStr"/>
     </row>
     <row r="16" ht="49.92" customHeight="1">
       <c r="A16" t="inlineStr">
@@ -4215,16 +4195,15 @@
       <c r="AL16" t="inlineStr"/>
       <c r="AM16" t="inlineStr"/>
       <c r="AN16" t="inlineStr"/>
-      <c r="AO16" t="inlineStr"/>
-      <c r="AP16" t="inlineStr">
+      <c r="AO16" t="inlineStr">
         <is>
           <t>Northport_church_BF</t>
         </is>
       </c>
+      <c r="AP16" t="inlineStr"/>
       <c r="AQ16" t="inlineStr"/>
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="inlineStr"/>
-      <c r="AT16" t="inlineStr"/>
     </row>
     <row r="17" ht="74.88" customHeight="1">
       <c r="A17" t="inlineStr">
@@ -4361,16 +4340,15 @@
         </is>
       </c>
       <c r="AN17" t="inlineStr"/>
-      <c r="AO17" t="inlineStr"/>
-      <c r="AP17" t="inlineStr">
+      <c r="AO17" t="inlineStr">
         <is>
           <t>Shinier_North</t>
         </is>
       </c>
+      <c r="AP17" t="inlineStr"/>
       <c r="AQ17" t="inlineStr"/>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="inlineStr"/>
-      <c r="AT17" t="inlineStr"/>
     </row>
     <row r="18" ht="74.10000000000001" customHeight="1">
       <c r="A18" t="inlineStr">
@@ -4507,16 +4485,15 @@
         </is>
       </c>
       <c r="AN18" t="inlineStr"/>
-      <c r="AO18" t="inlineStr"/>
-      <c r="AP18" t="inlineStr">
+      <c r="AO18" t="inlineStr">
         <is>
           <t>Shinier_North</t>
         </is>
       </c>
+      <c r="AP18" t="inlineStr"/>
       <c r="AQ18" t="inlineStr"/>
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="inlineStr"/>
-      <c r="AT18" t="inlineStr"/>
     </row>
     <row r="19" ht="42.12" customHeight="1">
       <c r="A19" t="inlineStr">
@@ -4653,16 +4630,15 @@
         </is>
       </c>
       <c r="AN19" t="inlineStr"/>
-      <c r="AO19" t="inlineStr"/>
-      <c r="AP19" t="inlineStr">
+      <c r="AO19" t="inlineStr">
         <is>
           <t>Shinier_North</t>
         </is>
       </c>
+      <c r="AP19" t="inlineStr"/>
       <c r="AQ19" t="inlineStr"/>
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="inlineStr"/>
-      <c r="AT19" t="inlineStr"/>
     </row>
     <row r="20" ht="74.88" customHeight="1">
       <c r="A20" t="inlineStr">
@@ -4799,16 +4775,15 @@
         </is>
       </c>
       <c r="AN20" t="inlineStr"/>
-      <c r="AO20" t="inlineStr"/>
-      <c r="AP20" t="inlineStr">
+      <c r="AO20" t="inlineStr">
         <is>
           <t>Shinier_North</t>
         </is>
       </c>
+      <c r="AP20" t="inlineStr"/>
       <c r="AQ20" t="inlineStr"/>
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="inlineStr"/>
-      <c r="AT20" t="inlineStr"/>
     </row>
     <row r="21" ht="51.48" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -4945,16 +4920,15 @@
         </is>
       </c>
       <c r="AN21" t="inlineStr"/>
-      <c r="AO21" t="inlineStr"/>
-      <c r="AP21" t="inlineStr">
+      <c r="AO21" t="inlineStr">
         <is>
           <t>Shinier_Wilds</t>
         </is>
       </c>
+      <c r="AP21" t="inlineStr"/>
       <c r="AQ21" t="inlineStr"/>
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="inlineStr"/>
-      <c r="AT21" t="inlineStr"/>
     </row>
     <row r="22" ht="74.88" customHeight="1">
       <c r="A22" t="inlineStr">
@@ -5091,16 +5065,15 @@
         </is>
       </c>
       <c r="AN22" t="inlineStr"/>
-      <c r="AO22" t="inlineStr"/>
-      <c r="AP22" t="inlineStr">
+      <c r="AO22" t="inlineStr">
         <is>
           <t>Shinier_Altar</t>
         </is>
       </c>
+      <c r="AP22" t="inlineStr"/>
       <c r="AQ22" t="inlineStr"/>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="inlineStr"/>
-      <c r="AT22" t="inlineStr"/>
     </row>
     <row r="23" ht="74.88" customHeight="1">
       <c r="A23" t="inlineStr">
@@ -5239,24 +5212,23 @@
         </is>
       </c>
       <c r="AN23" t="inlineStr"/>
-      <c r="AO23" t="inlineStr"/>
-      <c r="AP23" t="inlineStr">
+      <c r="AO23" t="inlineStr">
         <is>
           <t>Captal_Guild_Day</t>
         </is>
       </c>
-      <c r="AQ23" t="b">
-        <v>1</v>
-      </c>
-      <c r="AR23" t="n">
+      <c r="AP23" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ23" t="n">
         <v>5</v>
       </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>[{"id": "brass_casing", "n": 6}]</t>
+        </is>
+      </c>
       <c r="AS23" t="inlineStr">
-        <is>
-          <t>[{"id": "brass_casing", "n": 6}]</t>
-        </is>
-      </c>
-      <c r="AT23" t="inlineStr">
         <is>
           <t>{"hpRatio": [0.6, 0.8]}</t>
         </is>
@@ -5394,23 +5366,22 @@
       </c>
       <c r="AL24" t="inlineStr"/>
       <c r="AM24" t="inlineStr"/>
-      <c r="AN24" t="inlineStr"/>
-      <c r="AO24" t="b">
-        <v>1</v>
-      </c>
-      <c r="AP24" t="inlineStr"/>
-      <c r="AQ24" t="b">
-        <v>1</v>
-      </c>
-      <c r="AR24" t="n">
+      <c r="AN24" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO24" t="inlineStr"/>
+      <c r="AP24" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ24" t="n">
         <v>5</v>
       </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>[{"id": "venom_fang", "n": 1, "p": 0.1}, {"id": "venom_claw", "n": 1, "p": 0.33}, {"id": "chitin_wing", "n": 1, "p": 0.1}, {"id": "chitin_shell", "n": 1, "p": 0.33}]</t>
+        </is>
+      </c>
       <c r="AS24" t="inlineStr">
-        <is>
-          <t>[{"id": "venom_fang", "n": 1, "p": 0.1}, {"id": "venom_claw", "n": 1, "p": 0.33}, {"id": "chitin_wing", "n": 1, "p": 0.1}, {"id": "chitin_shell", "n": 1, "p": 0.33}]</t>
-        </is>
-      </c>
-      <c r="AT24" t="inlineStr">
         <is>
           <t>{"hpRatio": [1.2, 1.5]}</t>
         </is>
@@ -5550,23 +5521,22 @@
       </c>
       <c r="AL25" t="inlineStr"/>
       <c r="AM25" t="inlineStr"/>
-      <c r="AN25" t="inlineStr"/>
-      <c r="AO25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AP25" t="inlineStr"/>
-      <c r="AQ25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AR25" t="n">
+      <c r="AN25" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO25" t="inlineStr"/>
+      <c r="AP25" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ25" t="n">
         <v>5</v>
       </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>[{"id": "venom_fang", "n": 1, "p": 0.1}, {"id": "azure_scale", "n": 1, "p": 0.33}, {"id": "azure_feather", "n": 1, "p": 0.33}]</t>
+        </is>
+      </c>
       <c r="AS25" t="inlineStr">
-        <is>
-          <t>[{"id": "venom_fang", "n": 1, "p": 0.1}, {"id": "azure_scale", "n": 1, "p": 0.33}, {"id": "azure_feather", "n": 1, "p": 0.33}]</t>
-        </is>
-      </c>
-      <c r="AT25" t="inlineStr">
         <is>
           <t>{"hpRatio": [0.5, 0.7]}</t>
         </is>
@@ -5706,23 +5676,22 @@
       </c>
       <c r="AL26" t="inlineStr"/>
       <c r="AM26" t="inlineStr"/>
-      <c r="AN26" t="inlineStr"/>
-      <c r="AO26" t="b">
-        <v>1</v>
-      </c>
-      <c r="AP26" t="inlineStr"/>
-      <c r="AQ26" t="b">
-        <v>1</v>
-      </c>
-      <c r="AR26" t="n">
+      <c r="AN26" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO26" t="inlineStr"/>
+      <c r="AP26" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ26" t="n">
         <v>5</v>
       </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>[{"id": "brass_casing", "n": 1, "p": 0.33}]</t>
+        </is>
+      </c>
       <c r="AS26" t="inlineStr">
-        <is>
-          <t>[{"id": "brass_casing", "n": 1, "p": 0.33}]</t>
-        </is>
-      </c>
-      <c r="AT26" t="inlineStr">
         <is>
           <t>{"hpRatio": [0.7, 0.9]}</t>
         </is>
@@ -5863,20 +5832,19 @@
         </is>
       </c>
       <c r="AN27" t="inlineStr"/>
-      <c r="AO27" t="inlineStr"/>
-      <c r="AP27" t="inlineStr">
+      <c r="AO27" t="inlineStr">
         <is>
           <t>Forest_Glade_Day</t>
         </is>
       </c>
+      <c r="AP27" t="inlineStr"/>
       <c r="AQ27" t="inlineStr"/>
-      <c r="AR27" t="inlineStr"/>
-      <c r="AS27" t="inlineStr">
+      <c r="AR27" t="inlineStr">
         <is>
           <t>[{"id": "meat_lynx", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT27" t="inlineStr"/>
+      <c r="AS27" t="inlineStr"/>
     </row>
     <row r="28" ht="74.10000000000001" customHeight="1">
       <c r="A28" t="inlineStr">
@@ -6013,20 +5981,19 @@
         </is>
       </c>
       <c r="AN28" t="inlineStr"/>
-      <c r="AO28" t="inlineStr"/>
-      <c r="AP28" t="inlineStr">
+      <c r="AO28" t="inlineStr">
         <is>
           <t>Forest_Shoal_Day</t>
         </is>
       </c>
+      <c r="AP28" t="inlineStr"/>
       <c r="AQ28" t="inlineStr"/>
-      <c r="AR28" t="inlineStr"/>
-      <c r="AS28" t="inlineStr">
+      <c r="AR28" t="inlineStr">
         <is>
           <t>[{"id": "meat_snake", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT28" t="inlineStr"/>
+      <c r="AS28" t="inlineStr"/>
     </row>
     <row r="29" ht="33.54" customHeight="1">
       <c r="A29" t="inlineStr">
@@ -6163,20 +6130,19 @@
         </is>
       </c>
       <c r="AN29" t="inlineStr"/>
-      <c r="AO29" t="inlineStr"/>
-      <c r="AP29" t="inlineStr">
+      <c r="AO29" t="inlineStr">
         <is>
           <t>Forest_Trail_Day</t>
         </is>
       </c>
+      <c r="AP29" t="inlineStr"/>
       <c r="AQ29" t="inlineStr"/>
-      <c r="AR29" t="inlineStr"/>
-      <c r="AS29" t="inlineStr">
+      <c r="AR29" t="inlineStr">
         <is>
           <t>[{"id": "meat_boar", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT29" t="inlineStr"/>
+      <c r="AS29" t="inlineStr"/>
     </row>
     <row r="30" ht="33.54" customHeight="1">
       <c r="A30" t="inlineStr">
@@ -6313,20 +6279,19 @@
         </is>
       </c>
       <c r="AN30" t="inlineStr"/>
-      <c r="AO30" t="inlineStr"/>
-      <c r="AP30" t="inlineStr">
+      <c r="AO30" t="inlineStr">
         <is>
           <t>Forest_Cave_Day</t>
         </is>
       </c>
+      <c r="AP30" t="inlineStr"/>
       <c r="AQ30" t="inlineStr"/>
-      <c r="AR30" t="inlineStr"/>
-      <c r="AS30" t="inlineStr">
+      <c r="AR30" t="inlineStr">
         <is>
           <t>[{"id": "tiger_horn", "n": 1, "p": 0.25}]</t>
         </is>
       </c>
-      <c r="AT30" t="inlineStr"/>
+      <c r="AS30" t="inlineStr"/>
     </row>
     <row r="31" ht="74.88" customHeight="1">
       <c r="A31" t="inlineStr">
@@ -6463,20 +6428,19 @@
         </is>
       </c>
       <c r="AN31" t="inlineStr"/>
-      <c r="AO31" t="inlineStr"/>
-      <c r="AP31" t="inlineStr">
+      <c r="AO31" t="inlineStr">
         <is>
           <t>Forest_Glade_Day</t>
         </is>
       </c>
+      <c r="AP31" t="inlineStr"/>
       <c r="AQ31" t="inlineStr"/>
-      <c r="AR31" t="inlineStr"/>
-      <c r="AS31" t="inlineStr">
+      <c r="AR31" t="inlineStr">
         <is>
           <t>[{"id": "crow_beak", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT31" t="inlineStr"/>
+      <c r="AS31" t="inlineStr"/>
     </row>
     <row r="32" ht="53.04" customHeight="1">
       <c r="A32" t="inlineStr">
@@ -6613,20 +6577,19 @@
         </is>
       </c>
       <c r="AN32" t="inlineStr"/>
-      <c r="AO32" t="inlineStr"/>
-      <c r="AP32" t="inlineStr">
+      <c r="AO32" t="inlineStr">
         <is>
           <t>ruins_shinier_entrance</t>
         </is>
       </c>
+      <c r="AP32" t="inlineStr"/>
       <c r="AQ32" t="inlineStr"/>
-      <c r="AR32" t="inlineStr"/>
-      <c r="AS32" t="inlineStr">
+      <c r="AR32" t="inlineStr">
         <is>
           <t>[{"id": "elf_antler", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT32" t="inlineStr"/>
+      <c r="AS32" t="inlineStr"/>
     </row>
     <row r="33" ht="74.10000000000001" customHeight="1">
       <c r="A33" t="inlineStr">
@@ -6763,20 +6726,19 @@
         </is>
       </c>
       <c r="AN33" t="inlineStr"/>
-      <c r="AO33" t="inlineStr"/>
-      <c r="AP33" t="inlineStr">
+      <c r="AO33" t="inlineStr">
         <is>
           <t>Forest_Trail_Day</t>
         </is>
       </c>
+      <c r="AP33" t="inlineStr"/>
       <c r="AQ33" t="inlineStr"/>
-      <c r="AR33" t="inlineStr"/>
-      <c r="AS33" t="inlineStr">
+      <c r="AR33" t="inlineStr">
         <is>
           <t>[{"id": "paw_bear", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT33" t="inlineStr"/>
+      <c r="AS33" t="inlineStr"/>
     </row>
     <row r="34" ht="51.48" customHeight="1">
       <c r="A34" t="inlineStr">
@@ -6913,20 +6875,19 @@
         </is>
       </c>
       <c r="AN34" t="inlineStr"/>
-      <c r="AO34" t="inlineStr"/>
-      <c r="AP34" t="inlineStr">
+      <c r="AO34" t="inlineStr">
         <is>
           <t>Forest_Trail_Day</t>
         </is>
       </c>
+      <c r="AP34" t="inlineStr"/>
       <c r="AQ34" t="inlineStr"/>
-      <c r="AR34" t="inlineStr"/>
-      <c r="AS34" t="inlineStr">
+      <c r="AR34" t="inlineStr">
         <is>
           <t>[{"id": "paw_bear", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT34" t="inlineStr"/>
+      <c r="AS34" t="inlineStr"/>
     </row>
     <row r="35" ht="74.10000000000001" customHeight="1">
       <c r="A35" t="inlineStr">
@@ -7063,20 +7024,19 @@
         </is>
       </c>
       <c r="AN35" t="inlineStr"/>
-      <c r="AO35" t="inlineStr"/>
-      <c r="AP35" t="inlineStr">
+      <c r="AO35" t="inlineStr">
         <is>
           <t>Forest_Cliff_Day</t>
         </is>
       </c>
+      <c r="AP35" t="inlineStr"/>
       <c r="AQ35" t="inlineStr"/>
-      <c r="AR35" t="inlineStr"/>
-      <c r="AS35" t="inlineStr">
+      <c r="AR35" t="inlineStr">
         <is>
           <t>[{"id": "antler_deer", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT35" t="inlineStr"/>
+      <c r="AS35" t="inlineStr"/>
     </row>
     <row r="36" ht="42.12" customHeight="1">
       <c r="A36" t="inlineStr">
@@ -7213,20 +7173,19 @@
         </is>
       </c>
       <c r="AN36" t="inlineStr"/>
-      <c r="AO36" t="inlineStr"/>
-      <c r="AP36" t="inlineStr">
+      <c r="AO36" t="inlineStr">
         <is>
           <t>Forest_Cliff_Day</t>
         </is>
       </c>
+      <c r="AP36" t="inlineStr"/>
       <c r="AQ36" t="inlineStr"/>
-      <c r="AR36" t="inlineStr"/>
-      <c r="AS36" t="inlineStr">
+      <c r="AR36" t="inlineStr">
         <is>
           <t>[{"id": "antler_deer", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT36" t="inlineStr"/>
+      <c r="AS36" t="inlineStr"/>
     </row>
     <row r="37" ht="74.88" customHeight="1">
       <c r="A37" t="inlineStr">
@@ -7363,20 +7322,19 @@
         </is>
       </c>
       <c r="AN37" t="inlineStr"/>
-      <c r="AO37" t="inlineStr"/>
-      <c r="AP37" t="inlineStr">
+      <c r="AO37" t="inlineStr">
         <is>
           <t>Ruins_shinier_Catacomb</t>
         </is>
       </c>
+      <c r="AP37" t="inlineStr"/>
       <c r="AQ37" t="inlineStr"/>
-      <c r="AR37" t="inlineStr"/>
-      <c r="AS37" t="inlineStr">
+      <c r="AR37" t="inlineStr">
         <is>
           <t>[{"id": "harm_bone", "n": 1, "p": 0.1}]</t>
         </is>
       </c>
-      <c r="AT37" t="inlineStr"/>
+      <c r="AS37" t="inlineStr"/>
     </row>
     <row r="38" ht="74.88" customHeight="1">
       <c r="A38" t="inlineStr">
@@ -7513,20 +7471,19 @@
         </is>
       </c>
       <c r="AN38" t="inlineStr"/>
-      <c r="AO38" t="inlineStr"/>
-      <c r="AP38" t="inlineStr">
+      <c r="AO38" t="inlineStr">
         <is>
           <t>Ruins_shinier_Colossus</t>
         </is>
       </c>
+      <c r="AP38" t="inlineStr"/>
       <c r="AQ38" t="inlineStr"/>
-      <c r="AR38" t="inlineStr"/>
-      <c r="AS38" t="inlineStr">
+      <c r="AR38" t="inlineStr">
         <is>
           <t>[{"id": "bell_shard", "n": 1, "p": 0.1}]</t>
         </is>
       </c>
-      <c r="AT38" t="inlineStr"/>
+      <c r="AS38" t="inlineStr"/>
     </row>
     <row r="39" ht="74.88" customHeight="1">
       <c r="A39" t="inlineStr">
@@ -7663,20 +7620,19 @@
         </is>
       </c>
       <c r="AN39" t="inlineStr"/>
-      <c r="AO39" t="inlineStr"/>
-      <c r="AP39" t="inlineStr">
+      <c r="AO39" t="inlineStr">
         <is>
           <t>Ruins_shinier_Hollow</t>
         </is>
       </c>
+      <c r="AP39" t="inlineStr"/>
       <c r="AQ39" t="inlineStr"/>
-      <c r="AR39" t="inlineStr"/>
-      <c r="AS39" t="inlineStr">
+      <c r="AR39" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AT39" t="inlineStr"/>
+      <c r="AS39" t="inlineStr"/>
     </row>
     <row r="40" ht="74.88" customHeight="1">
       <c r="A40" t="inlineStr">
@@ -7813,20 +7769,19 @@
         </is>
       </c>
       <c r="AN40" t="inlineStr"/>
-      <c r="AO40" t="inlineStr"/>
-      <c r="AP40" t="inlineStr">
+      <c r="AO40" t="inlineStr">
         <is>
           <t>Ruins_shinier_Prison</t>
         </is>
       </c>
+      <c r="AP40" t="inlineStr"/>
       <c r="AQ40" t="inlineStr"/>
-      <c r="AR40" t="inlineStr"/>
-      <c r="AS40" t="inlineStr">
+      <c r="AR40" t="inlineStr">
         <is>
           <t>[{"id": "harm_claw", "n": 1, "p": 0.1}]</t>
         </is>
       </c>
-      <c r="AT40" t="inlineStr"/>
+      <c r="AS40" t="inlineStr"/>
     </row>
     <row r="41" ht="74.10000000000001" customHeight="1">
       <c r="A41" t="inlineStr">
@@ -7963,20 +7918,19 @@
         </is>
       </c>
       <c r="AN41" t="inlineStr"/>
-      <c r="AO41" t="inlineStr"/>
-      <c r="AP41" t="inlineStr">
+      <c r="AO41" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP41" t="inlineStr"/>
       <c r="AQ41" t="inlineStr"/>
-      <c r="AR41" t="inlineStr"/>
-      <c r="AS41" t="inlineStr">
+      <c r="AR41" t="inlineStr">
         <is>
           <t>[{"id": "bell_shard", "n": 1, "p": 0.1}]</t>
         </is>
       </c>
-      <c r="AT41" t="inlineStr"/>
+      <c r="AS41" t="inlineStr"/>
     </row>
     <row r="42" ht="74.88" customHeight="1">
       <c r="A42" t="inlineStr">
@@ -8113,20 +8067,19 @@
         </is>
       </c>
       <c r="AN42" t="inlineStr"/>
-      <c r="AO42" t="inlineStr"/>
-      <c r="AP42" t="inlineStr">
+      <c r="AO42" t="inlineStr">
         <is>
           <t>Ruins_shinier_Prison</t>
         </is>
       </c>
+      <c r="AP42" t="inlineStr"/>
       <c r="AQ42" t="inlineStr"/>
-      <c r="AR42" t="inlineStr"/>
-      <c r="AS42" t="inlineStr">
+      <c r="AR42" t="inlineStr">
         <is>
           <t>[{"id": "saint_claw", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT42" t="inlineStr"/>
+      <c r="AS42" t="inlineStr"/>
     </row>
     <row r="43" ht="74.88" customHeight="1">
       <c r="A43" t="inlineStr">
@@ -8263,20 +8216,19 @@
         </is>
       </c>
       <c r="AN43" t="inlineStr"/>
-      <c r="AO43" t="inlineStr"/>
-      <c r="AP43" t="inlineStr">
+      <c r="AO43" t="inlineStr">
         <is>
           <t>Ruins_shinier_DarkBridge</t>
         </is>
       </c>
+      <c r="AP43" t="inlineStr"/>
       <c r="AQ43" t="inlineStr"/>
-      <c r="AR43" t="inlineStr"/>
-      <c r="AS43" t="inlineStr">
+      <c r="AR43" t="inlineStr">
         <is>
           <t>[{"id": "saint_fang", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT43" t="inlineStr"/>
+      <c r="AS43" t="inlineStr"/>
     </row>
     <row r="44" ht="74.88" customHeight="1">
       <c r="A44" t="inlineStr">
@@ -8413,20 +8365,19 @@
         </is>
       </c>
       <c r="AN44" t="inlineStr"/>
-      <c r="AO44" t="inlineStr"/>
-      <c r="AP44" t="inlineStr">
+      <c r="AO44" t="inlineStr">
         <is>
           <t>Ruins_shinier_CorridorA</t>
         </is>
       </c>
+      <c r="AP44" t="inlineStr"/>
       <c r="AQ44" t="inlineStr"/>
-      <c r="AR44" t="inlineStr"/>
-      <c r="AS44" t="inlineStr">
+      <c r="AR44" t="inlineStr">
         <is>
           <t>[{"id": "saint_bone_big", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT44" t="inlineStr"/>
+      <c r="AS44" t="inlineStr"/>
     </row>
     <row r="45" ht="74.88" customHeight="1">
       <c r="A45" t="inlineStr">
@@ -8563,20 +8514,19 @@
         </is>
       </c>
       <c r="AN45" t="inlineStr"/>
-      <c r="AO45" t="inlineStr"/>
-      <c r="AP45" t="inlineStr">
+      <c r="AO45" t="inlineStr">
         <is>
           <t>Ruins_shinier_DeepAltar</t>
         </is>
       </c>
+      <c r="AP45" t="inlineStr"/>
       <c r="AQ45" t="inlineStr"/>
-      <c r="AR45" t="inlineStr"/>
-      <c r="AS45" t="inlineStr">
+      <c r="AR45" t="inlineStr">
         <is>
           <t>[{"id": "saint_bone", "n": 1}]</t>
         </is>
       </c>
-      <c r="AT45" t="inlineStr"/>
+      <c r="AS45" t="inlineStr"/>
     </row>
     <row r="46" ht="74.88" customHeight="1">
       <c r="A46" t="inlineStr">
@@ -8713,16 +8663,15 @@
         </is>
       </c>
       <c r="AN46" t="inlineStr"/>
-      <c r="AO46" t="inlineStr"/>
-      <c r="AP46" t="inlineStr">
+      <c r="AO46" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP46" t="inlineStr"/>
       <c r="AQ46" t="inlineStr"/>
       <c r="AR46" t="inlineStr"/>
       <c r="AS46" t="inlineStr"/>
-      <c r="AT46" t="inlineStr"/>
     </row>
     <row r="47" ht="74.88" customHeight="1">
       <c r="A47" t="inlineStr">
@@ -8859,16 +8808,15 @@
         </is>
       </c>
       <c r="AN47" t="inlineStr"/>
-      <c r="AO47" t="inlineStr"/>
-      <c r="AP47" t="inlineStr">
+      <c r="AO47" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP47" t="inlineStr"/>
       <c r="AQ47" t="inlineStr"/>
       <c r="AR47" t="inlineStr"/>
       <c r="AS47" t="inlineStr"/>
-      <c r="AT47" t="inlineStr"/>
     </row>
     <row r="48" ht="74.88" customHeight="1">
       <c r="A48" t="inlineStr">
@@ -9005,16 +8953,15 @@
         </is>
       </c>
       <c r="AN48" t="inlineStr"/>
-      <c r="AO48" t="inlineStr"/>
-      <c r="AP48" t="inlineStr">
+      <c r="AO48" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP48" t="inlineStr"/>
       <c r="AQ48" t="inlineStr"/>
       <c r="AR48" t="inlineStr"/>
       <c r="AS48" t="inlineStr"/>
-      <c r="AT48" t="inlineStr"/>
     </row>
     <row r="49" ht="74.88" customHeight="1">
       <c r="A49" t="inlineStr">
@@ -9151,16 +9098,15 @@
         </is>
       </c>
       <c r="AN49" t="inlineStr"/>
-      <c r="AO49" t="inlineStr"/>
-      <c r="AP49" t="inlineStr">
+      <c r="AO49" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP49" t="inlineStr"/>
       <c r="AQ49" t="inlineStr"/>
       <c r="AR49" t="inlineStr"/>
       <c r="AS49" t="inlineStr"/>
-      <c r="AT49" t="inlineStr"/>
     </row>
     <row r="50" ht="74.88" customHeight="1">
       <c r="A50" t="inlineStr">
@@ -9297,16 +9243,15 @@
         </is>
       </c>
       <c r="AN50" t="inlineStr"/>
-      <c r="AO50" t="inlineStr"/>
-      <c r="AP50" t="inlineStr">
+      <c r="AO50" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP50" t="inlineStr"/>
       <c r="AQ50" t="inlineStr"/>
       <c r="AR50" t="inlineStr"/>
       <c r="AS50" t="inlineStr"/>
-      <c r="AT50" t="inlineStr"/>
     </row>
     <row r="51" ht="74.88" customHeight="1">
       <c r="A51" t="inlineStr">
@@ -9443,16 +9388,15 @@
         </is>
       </c>
       <c r="AN51" t="inlineStr"/>
-      <c r="AO51" t="inlineStr"/>
-      <c r="AP51" t="inlineStr">
+      <c r="AO51" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP51" t="inlineStr"/>
       <c r="AQ51" t="inlineStr"/>
       <c r="AR51" t="inlineStr"/>
       <c r="AS51" t="inlineStr"/>
-      <c r="AT51" t="inlineStr"/>
     </row>
     <row r="52" ht="74.88" customHeight="1">
       <c r="A52" t="inlineStr">
@@ -9589,16 +9533,15 @@
         </is>
       </c>
       <c r="AN52" t="inlineStr"/>
-      <c r="AO52" t="inlineStr"/>
-      <c r="AP52" t="inlineStr">
+      <c r="AO52" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP52" t="inlineStr"/>
       <c r="AQ52" t="inlineStr"/>
       <c r="AR52" t="inlineStr"/>
       <c r="AS52" t="inlineStr"/>
-      <c r="AT52" t="inlineStr"/>
     </row>
     <row r="53" ht="74.88" customHeight="1">
       <c r="A53" t="inlineStr">
@@ -9735,16 +9678,15 @@
         </is>
       </c>
       <c r="AN53" t="inlineStr"/>
-      <c r="AO53" t="inlineStr"/>
-      <c r="AP53" t="inlineStr">
+      <c r="AO53" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP53" t="inlineStr"/>
       <c r="AQ53" t="inlineStr"/>
       <c r="AR53" t="inlineStr"/>
       <c r="AS53" t="inlineStr"/>
-      <c r="AT53" t="inlineStr"/>
     </row>
     <row r="54" ht="74.88" customHeight="1">
       <c r="A54" t="inlineStr">
@@ -9881,16 +9823,15 @@
         </is>
       </c>
       <c r="AN54" t="inlineStr"/>
-      <c r="AO54" t="inlineStr"/>
-      <c r="AP54" t="inlineStr">
+      <c r="AO54" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP54" t="inlineStr"/>
       <c r="AQ54" t="inlineStr"/>
       <c r="AR54" t="inlineStr"/>
       <c r="AS54" t="inlineStr"/>
-      <c r="AT54" t="inlineStr"/>
     </row>
     <row r="55" ht="74.88" customHeight="1">
       <c r="A55" t="inlineStr">
@@ -10027,16 +9968,15 @@
         </is>
       </c>
       <c r="AN55" t="inlineStr"/>
-      <c r="AO55" t="inlineStr"/>
-      <c r="AP55" t="inlineStr">
+      <c r="AO55" t="inlineStr">
         <is>
           <t>Ruins_shinier_MossChamber</t>
         </is>
       </c>
+      <c r="AP55" t="inlineStr"/>
       <c r="AQ55" t="inlineStr"/>
       <c r="AR55" t="inlineStr"/>
       <c r="AS55" t="inlineStr"/>
-      <c r="AT55" t="inlineStr"/>
     </row>
     <row r="56" ht="74.88" customHeight="1">
       <c r="A56" t="inlineStr"/>
@@ -10088,7 +10028,6 @@
       <c r="AQ56" t="inlineStr"/>
       <c r="AR56" t="inlineStr"/>
       <c r="AS56" t="inlineStr"/>
-      <c r="AT56" t="inlineStr"/>
     </row>
     <row r="57" ht="74.88" customHeight="1">
       <c r="A57" t="inlineStr"/>
@@ -10140,7 +10079,6 @@
       <c r="AQ57" t="inlineStr"/>
       <c r="AR57" t="inlineStr"/>
       <c r="AS57" t="inlineStr"/>
-      <c r="AT57" t="inlineStr"/>
     </row>
     <row r="58" ht="74.88" customHeight="1">
       <c r="A58" t="inlineStr"/>
@@ -10192,7 +10130,6 @@
       <c r="AQ58" t="inlineStr"/>
       <c r="AR58" t="inlineStr"/>
       <c r="AS58" t="inlineStr"/>
-      <c r="AT58" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10217,7 +10154,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>48fce4d0cc9b8e0e46596adbd555eb6ea414f7e878f93e135e2d78e7f9cf6ce1</t>
+          <t>6d44766f52cbb7f4569199cae7007a757a0d261a2b92fac9370c0554b610dc59</t>
         </is>
       </c>
     </row>

</xml_diff>